<commit_message>
Fix bug with squad name in excel workbook dashboard
</commit_message>
<xml_diff>
--- a/assets/xlsx/visualise-metrics.xlsx
+++ b/assets/xlsx/visualise-metrics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/workspace/sprint-metrics_webapp/steps/visualise-metrics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4E5D8E-E245-544B-B021-B52E37DFDA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA97840B-3A3D-6A4C-BCFF-85C5F38583D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="157">
   <si>
     <t>Done</t>
   </si>
@@ -572,29 +572,23 @@
     <t>metricConfidence_totalUnestimatedWorkitems</t>
   </si>
   <si>
-    <t>m</t>
+    <t>Project</t>
   </si>
   <si>
-    <t>Project1</t>
+    <t>Cloud</t>
   </si>
   <si>
-    <t>Project2</t>
+    <t>Dataverse</t>
   </si>
   <si>
-    <t>StreamA</t>
-  </si>
-  <si>
-    <t>StreamB</t>
-  </si>
-  <si>
-    <t>StreamC</t>
+    <t>Architecture</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -736,6 +730,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="30">
@@ -1231,7 +1238,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1434,7 +1441,6 @@
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1507,6 +1513,9 @@
     <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
@@ -1920,10 +1929,10 @@
                   <c:v>BAU/Improvement</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Project1</c:v>
+                  <c:v>Convergence</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Project2</c:v>
+                  <c:v>Project</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3270,13 +3279,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>StreamA</c:v>
+                  <c:v>Cloud</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>StreamB</c:v>
+                  <c:v>Dataverse</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>StreamC</c:v>
+                  <c:v>Architecture</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -7976,7 +7985,7 @@
       <xdr:row>2</xdr:row>
       <xdr:rowOff>1637676</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="#REF!">
+    <xdr:sp macro="" textlink="'Sprint Summary | data'!B5">
       <xdr:nvSpPr>
         <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
@@ -8018,7 +8027,7 @@
         <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
         <a:lstStyle/>
         <a:p>
-          <a:fld id="{05B068DF-ADDA-448C-9145-DA3574541357}" type="TxLink">
+          <a:fld id="{DC27AAE4-6848-F34A-B44F-24CDDF2D445C}" type="TxLink">
             <a:rPr lang="en-US" sz="3200" b="0" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:schemeClr val="bg2">
@@ -8028,8 +8037,7 @@
               <a:latin typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
-            <a:pPr/>
-            <a:t>Architecture &amp; Engineering</a:t>
+            <a:t>0</a:t>
           </a:fld>
           <a:endParaRPr lang="en-AU" sz="3200" b="1">
             <a:solidFill>
@@ -13759,7 +13767,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>Project1</a:t>
+                <a:t>Convergence</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -14088,7 +14096,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>Project2</a:t>
+                <a:t>Project</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -15393,7 +15401,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>StreamA</a:t>
+                <a:t>Cloud</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -15722,7 +15730,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>StreamB</a:t>
+                <a:t>Dataverse</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -16048,7 +16056,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>StreamC</a:t>
+                <a:t>Architecture</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -20155,7 +20163,7 @@
   <sheetPr>
     <tabColor rgb="FF006600"/>
   </sheetPr>
-  <dimension ref="B1:R16"/>
+  <dimension ref="B1:M16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="32" customWidth="1"/>
@@ -20174,8 +20182,8 @@
     <col min="14" max="16384" width="8.6640625" style="32"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" ht="42.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:18" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:13" ht="42.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:13" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="31"/>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
@@ -20189,56 +20197,53 @@
       <c r="L2" s="31"/>
       <c r="M2" s="31"/>
     </row>
-    <row r="3" spans="2:18" ht="137" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" ht="137" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="31"/>
-      <c r="C3" s="111"/>
-      <c r="D3" s="112"/>
-      <c r="E3" s="112"/>
-      <c r="F3" s="112"/>
-      <c r="G3" s="112"/>
-      <c r="H3" s="112"/>
-      <c r="I3" s="112"/>
-      <c r="J3" s="112"/>
-      <c r="K3" s="112"/>
-      <c r="L3" s="112"/>
+      <c r="C3" s="110"/>
+      <c r="D3" s="111"/>
+      <c r="E3" s="111"/>
+      <c r="F3" s="111"/>
+      <c r="G3" s="111"/>
+      <c r="H3" s="111"/>
+      <c r="I3" s="111"/>
+      <c r="J3" s="111"/>
+      <c r="K3" s="111"/>
+      <c r="L3" s="111"/>
       <c r="M3" s="36"/>
     </row>
-    <row r="4" spans="2:18" ht="243.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:13" ht="243.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="31"/>
       <c r="C4" s="29"/>
-      <c r="D4" s="118"/>
-      <c r="E4" s="119"/>
-      <c r="F4" s="125"/>
-      <c r="G4" s="125"/>
-      <c r="H4" s="125"/>
-      <c r="I4" s="126"/>
-      <c r="J4" s="124"/>
-      <c r="K4" s="125"/>
-      <c r="L4" s="126"/>
+      <c r="D4" s="117"/>
+      <c r="E4" s="118"/>
+      <c r="F4" s="124"/>
+      <c r="G4" s="124"/>
+      <c r="H4" s="124"/>
+      <c r="I4" s="125"/>
+      <c r="J4" s="123"/>
+      <c r="K4" s="124"/>
+      <c r="L4" s="125"/>
       <c r="M4" s="31"/>
-      <c r="R4" s="32" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="2:18" ht="226.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="2:13" ht="226.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="31"/>
       <c r="C5" s="30"/>
       <c r="D5" s="48"/>
       <c r="E5" s="49"/>
-      <c r="F5" s="113"/>
-      <c r="G5" s="114"/>
-      <c r="H5" s="114"/>
-      <c r="I5" s="115"/>
-      <c r="J5" s="113"/>
-      <c r="K5" s="114"/>
-      <c r="L5" s="115"/>
+      <c r="F5" s="112"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="113"/>
+      <c r="I5" s="114"/>
+      <c r="J5" s="112"/>
+      <c r="K5" s="113"/>
+      <c r="L5" s="114"/>
       <c r="M5" s="31"/>
     </row>
-    <row r="6" spans="2:18" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:13" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="31"/>
-      <c r="C6" s="116"/>
-      <c r="D6" s="120"/>
-      <c r="E6" s="121"/>
+      <c r="C6" s="115"/>
+      <c r="D6" s="119"/>
+      <c r="E6" s="120"/>
       <c r="F6" s="35"/>
       <c r="G6" s="37"/>
       <c r="H6" s="38"/>
@@ -20248,29 +20253,29 @@
       <c r="L6" s="39"/>
       <c r="M6" s="31"/>
     </row>
-    <row r="7" spans="2:18" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:13" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="31"/>
-      <c r="C7" s="117"/>
-      <c r="D7" s="111"/>
-      <c r="E7" s="112"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="110"/>
+      <c r="E7" s="111"/>
       <c r="F7" s="34"/>
       <c r="G7" s="44"/>
-      <c r="H7" s="127" t="s">
+      <c r="H7" s="126" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="127"/>
-      <c r="J7" s="127" t="s">
+      <c r="I7" s="126"/>
+      <c r="J7" s="126" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="127"/>
+      <c r="K7" s="126"/>
       <c r="L7" s="40"/>
       <c r="M7" s="31"/>
     </row>
-    <row r="8" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="31"/>
-      <c r="C8" s="117"/>
-      <c r="D8" s="111"/>
-      <c r="E8" s="112"/>
+      <c r="C8" s="116"/>
+      <c r="D8" s="110"/>
+      <c r="E8" s="111"/>
       <c r="F8" s="34"/>
       <c r="G8" s="46" t="s">
         <v>9</v>
@@ -20294,11 +20299,11 @@
       <c r="L8" s="40"/>
       <c r="M8" s="31"/>
     </row>
-    <row r="9" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="31"/>
-      <c r="C9" s="117"/>
-      <c r="D9" s="111"/>
-      <c r="E9" s="112"/>
+      <c r="C9" s="116"/>
+      <c r="D9" s="110"/>
+      <c r="E9" s="111"/>
       <c r="F9" s="34"/>
       <c r="G9" s="50" t="s">
         <v>10</v>
@@ -20325,11 +20330,11 @@
       </c>
       <c r="M9" s="31"/>
     </row>
-    <row r="10" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="31"/>
-      <c r="C10" s="117"/>
-      <c r="D10" s="111"/>
-      <c r="E10" s="112"/>
+      <c r="C10" s="116"/>
+      <c r="D10" s="110"/>
+      <c r="E10" s="111"/>
       <c r="F10" s="34"/>
       <c r="G10" s="51" t="s">
         <v>56</v>
@@ -20356,11 +20361,11 @@
       </c>
       <c r="M10" s="31"/>
     </row>
-    <row r="11" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="31"/>
-      <c r="C11" s="117"/>
-      <c r="D11" s="111"/>
-      <c r="E11" s="112"/>
+      <c r="C11" s="116"/>
+      <c r="D11" s="110"/>
+      <c r="E11" s="111"/>
       <c r="F11" s="34"/>
       <c r="G11" s="46" t="s">
         <v>59</v>
@@ -20384,11 +20389,11 @@
       <c r="L11" s="40"/>
       <c r="M11" s="31"/>
     </row>
-    <row r="12" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="31"/>
-      <c r="C12" s="117"/>
-      <c r="D12" s="111"/>
-      <c r="E12" s="112"/>
+      <c r="C12" s="116"/>
+      <c r="D12" s="110"/>
+      <c r="E12" s="111"/>
       <c r="F12" s="34"/>
       <c r="G12" s="46" t="s">
         <v>57</v>
@@ -20412,11 +20417,11 @@
       <c r="L12" s="40"/>
       <c r="M12" s="31"/>
     </row>
-    <row r="13" spans="2:18" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="31"/>
-      <c r="C13" s="117"/>
-      <c r="D13" s="111"/>
-      <c r="E13" s="112"/>
+      <c r="C13" s="116"/>
+      <c r="D13" s="110"/>
+      <c r="E13" s="111"/>
       <c r="F13" s="34"/>
       <c r="G13" s="46" t="s">
         <v>58</v>
@@ -20440,11 +20445,11 @@
       <c r="L13" s="40"/>
       <c r="M13" s="31"/>
     </row>
-    <row r="14" spans="2:18" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="31"/>
-      <c r="C14" s="117"/>
-      <c r="D14" s="122"/>
-      <c r="E14" s="123"/>
+      <c r="C14" s="116"/>
+      <c r="D14" s="121"/>
+      <c r="E14" s="122"/>
       <c r="F14" s="33"/>
       <c r="G14" s="41"/>
       <c r="H14" s="42"/>
@@ -20454,21 +20459,21 @@
       <c r="L14" s="43"/>
       <c r="M14" s="31"/>
     </row>
-    <row r="15" spans="2:18" ht="264.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" ht="264.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B15" s="31"/>
-      <c r="C15" s="117"/>
-      <c r="D15" s="118"/>
-      <c r="E15" s="119"/>
-      <c r="F15" s="113"/>
-      <c r="G15" s="114"/>
-      <c r="H15" s="114"/>
-      <c r="I15" s="114"/>
-      <c r="J15" s="114"/>
-      <c r="K15" s="114"/>
-      <c r="L15" s="115"/>
+      <c r="C15" s="116"/>
+      <c r="D15" s="117"/>
+      <c r="E15" s="118"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="113"/>
+      <c r="H15" s="113"/>
+      <c r="I15" s="113"/>
+      <c r="J15" s="113"/>
+      <c r="K15" s="113"/>
+      <c r="L15" s="114"/>
       <c r="M15" s="36"/>
     </row>
-    <row r="16" spans="2:18" ht="10" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:13" ht="10" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="31"/>
       <c r="C16" s="31"/>
       <c r="D16" s="31"/>
@@ -20590,8 +20595,13 @@
       <c r="X4"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B5" s="4">
+        <f>'Calculated Stats'!C22</f>
+        <v>0</v>
+      </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
@@ -21224,7 +21234,7 @@
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Project1</v>
+        <v>Convergence</v>
       </c>
       <c r="B30" s="54">
         <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A30, 'Calculated Stats'!B$36:B$45, 0))</f>
@@ -21256,7 +21266,7 @@
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project2</v>
+        <v>Project</v>
       </c>
       <c r="B31" s="54">
         <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A31, 'Calculated Stats'!B$36:B$45, 0))</f>
@@ -21401,7 +21411,7 @@
       <c r="O40" s="4"/>
       <c r="Q40" s="4" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>StreamA</v>
+        <v>Cloud</v>
       </c>
       <c r="R40" s="4">
         <f>INDEX('Calculated Stats'!D$66:D$75, MATCH(Q40, 'Calculated Stats'!B$66:B$75, 0))</f>
@@ -21430,7 +21440,7 @@
       <c r="O41" s="4"/>
       <c r="Q41" s="4" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>StreamB</v>
+        <v>Dataverse</v>
       </c>
       <c r="R41" s="4">
         <f>INDEX('Calculated Stats'!D$66:D$75, MATCH(Q41, 'Calculated Stats'!B$66:B$75, 0))</f>
@@ -21455,7 +21465,7 @@
       <c r="O42" s="4"/>
       <c r="Q42" s="4" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>StreamC</v>
+        <v>Architecture</v>
       </c>
       <c r="R42" s="4">
         <f>INDEX('Calculated Stats'!D$66:D$75, MATCH(Q42, 'Calculated Stats'!B$66:B$75, 0))</f>
@@ -21907,10 +21917,10 @@
       <c r="G5" s="105"/>
     </row>
     <row r="6" spans="2:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="128" t="s">
+      <c r="B6" s="127" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="129"/>
+      <c r="C6" s="128"/>
       <c r="D6" s="105"/>
       <c r="E6" s="105"/>
       <c r="F6" s="106"/>
@@ -21933,7 +21943,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="79" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D8" s="105"/>
       <c r="E8" s="105"/>
@@ -21945,7 +21955,7 @@
         <v>53</v>
       </c>
       <c r="C9" s="79" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D9" s="105"/>
       <c r="E9" s="105"/>
@@ -21954,10 +21964,10 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="76" t="s">
-        <v>154</v>
+        <v>2</v>
       </c>
       <c r="C10" s="79" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D10" s="105"/>
       <c r="E10" s="105"/>
@@ -21966,7 +21976,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="76" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C11" s="79"/>
       <c r="D11" s="105"/>
@@ -22181,10 +22191,10 @@
       <c r="G31" s="105"/>
     </row>
     <row r="32" spans="2:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="128" t="s">
+      <c r="B32" s="127" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="129"/>
+      <c r="C32" s="128"/>
       <c r="D32" s="28"/>
       <c r="E32" s="28"/>
       <c r="F32" s="94"/>
@@ -22203,10 +22213,10 @@
       <c r="B34" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="133" t="s">
+      <c r="C34" s="132" t="s">
         <v>5</v>
       </c>
-      <c r="D34" s="133"/>
+      <c r="D34" s="132"/>
       <c r="E34" s="105"/>
       <c r="F34" s="105"/>
       <c r="G34" s="104"/>
@@ -22266,7 +22276,7 @@
     <row r="38" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B38" s="82" t="str">
         <f t="shared" si="0"/>
-        <v>Project1</v>
+        <v>Convergence</v>
       </c>
       <c r="C38" s="4">
         <f>'processed | data'!B19</f>
@@ -22284,7 +22294,7 @@
     <row r="39" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B39" s="82" t="str">
         <f t="shared" si="0"/>
-        <v>Project2</v>
+        <v>Project</v>
       </c>
       <c r="C39" s="4">
         <f>'processed | data'!B20</f>
@@ -22438,10 +22448,10 @@
       <c r="B49" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C49" s="133" t="s">
+      <c r="C49" s="132" t="s">
         <v>83</v>
       </c>
-      <c r="D49" s="133"/>
+      <c r="D49" s="132"/>
       <c r="E49" s="105"/>
       <c r="F49" s="105"/>
       <c r="G49" s="105"/>
@@ -22501,7 +22511,7 @@
     <row r="53" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B53" s="82" t="str">
         <f t="shared" si="1"/>
-        <v>Project1</v>
+        <v>Convergence</v>
       </c>
       <c r="C53" s="4">
         <f>'processed | data'!B70</f>
@@ -22519,7 +22529,7 @@
     <row r="54" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B54" s="82" t="str">
         <f t="shared" si="1"/>
-        <v>Project2</v>
+        <v>Project</v>
       </c>
       <c r="C54" s="4">
         <f>'processed | data'!B71</f>
@@ -22673,10 +22683,10 @@
       <c r="B64" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C64" s="134" t="s">
+      <c r="C64" s="133" t="s">
         <v>5</v>
       </c>
-      <c r="D64" s="134"/>
+      <c r="D64" s="133"/>
       <c r="E64" s="105"/>
       <c r="F64" s="105"/>
       <c r="G64" s="105"/>
@@ -22700,7 +22710,7 @@
     <row r="66" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B66" s="82" t="str">
         <f>C8</f>
-        <v>StreamA</v>
+        <v>Cloud</v>
       </c>
       <c r="C66" s="101">
         <f>'processed | data'!B41</f>
@@ -22718,7 +22728,7 @@
     <row r="67" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B67" s="82" t="str">
         <f t="shared" ref="B67:B75" si="2">C9</f>
-        <v>StreamB</v>
+        <v>Dataverse</v>
       </c>
       <c r="C67" s="101">
         <f>'processed | data'!B42</f>
@@ -22736,7 +22746,7 @@
     <row r="68" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B68" s="82" t="str">
         <f t="shared" si="2"/>
-        <v>StreamC</v>
+        <v>Architecture</v>
       </c>
       <c r="C68" s="101">
         <f>'processed | data'!B43</f>
@@ -22908,10 +22918,10 @@
       <c r="B79" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C79" s="134" t="s">
+      <c r="C79" s="133" t="s">
         <v>83</v>
       </c>
-      <c r="D79" s="134"/>
+      <c r="D79" s="133"/>
       <c r="E79" s="105"/>
       <c r="F79" s="105"/>
       <c r="G79" s="105"/>
@@ -22935,7 +22945,7 @@
     <row r="81" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B81" s="82" t="str">
         <f>C8</f>
-        <v>StreamA</v>
+        <v>Cloud</v>
       </c>
       <c r="C81" s="101">
         <f>'processed | data'!B92</f>
@@ -22953,7 +22963,7 @@
     <row r="82" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B82" s="82" t="str">
         <f t="shared" ref="B82:B90" si="3">C9</f>
-        <v>StreamB</v>
+        <v>Dataverse</v>
       </c>
       <c r="C82" s="101">
         <f>'processed | data'!B93</f>
@@ -22971,7 +22981,7 @@
     <row r="83" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B83" s="82" t="str">
         <f t="shared" si="3"/>
-        <v>StreamC</v>
+        <v>Architecture</v>
       </c>
       <c r="C83" s="101">
         <f>'processed | data'!B94</f>
@@ -23294,14 +23304,14 @@
     </row>
     <row r="104" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B104" s="6"/>
-      <c r="C104" s="130" t="s">
+      <c r="C104" s="129" t="s">
         <v>6</v>
       </c>
-      <c r="D104" s="131"/>
-      <c r="E104" s="130" t="s">
+      <c r="D104" s="130"/>
+      <c r="E104" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="F104" s="132"/>
+      <c r="F104" s="131"/>
       <c r="G104" s="6"/>
       <c r="N104" s="107"/>
     </row>
@@ -24729,7 +24739,7 @@
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Project1</v>
+        <v>Convergence</v>
       </c>
       <c r="B19" s="53" cm="1">
         <f t="array" ref="B19">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E19), 0)</f>
@@ -24737,7 +24747,7 @@
       </c>
       <c r="D19" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A19,"_",D$15)</f>
-        <v>labels_Project1_storyPoints</v>
+        <v>labels_Convergence_storyPoints</v>
       </c>
       <c r="E19" s="68" t="e">
         <f>MATCH(D19, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -24747,7 +24757,7 @@
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project2</v>
+        <v>Project</v>
       </c>
       <c r="B20" s="53" cm="1">
         <f t="array" ref="B20">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E20), 0)</f>
@@ -24755,7 +24765,7 @@
       </c>
       <c r="D20" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A20, "_",D$15)</f>
-        <v>labels_Project2_storyPoints</v>
+        <v>labels_Project_storyPoints</v>
       </c>
       <c r="E20" s="68" t="e">
         <f>MATCH(D20, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -24926,7 +24936,7 @@
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Project1</v>
+        <v>Convergence</v>
       </c>
       <c r="B31" s="53" cm="1">
         <f t="array" ref="B31">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E31), 0)</f>
@@ -24934,7 +24944,7 @@
       </c>
       <c r="D31" s="68" t="str">
         <f t="shared" si="0"/>
-        <v>completedLabels_Project1_storyPoints</v>
+        <v>completedLabels_Convergence_storyPoints</v>
       </c>
       <c r="E31" s="68" t="e">
         <f>MATCH(D31, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -24944,7 +24954,7 @@
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project2</v>
+        <v>Project</v>
       </c>
       <c r="B32" s="53" cm="1">
         <f t="array" ref="B32">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E32), 0)</f>
@@ -24952,7 +24962,7 @@
       </c>
       <c r="D32" s="68" t="str">
         <f t="shared" si="0"/>
-        <v>completedLabels_Project2_storyPoints</v>
+        <v>completedLabels_Project_storyPoints</v>
       </c>
       <c r="E32" s="68" t="e">
         <f>MATCH(D32, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25087,7 +25097,7 @@
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>StreamA</v>
+        <v>Cloud</v>
       </c>
       <c r="B41" s="88" cm="1">
         <f t="array" ref="B41">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E41), 0)</f>
@@ -25095,7 +25105,7 @@
       </c>
       <c r="D41" s="68" t="str">
         <f t="shared" ref="D41:D50" si="1">_xlfn.CONCAT("components_", A41,"_",D$15)</f>
-        <v>components_StreamA_storyPoints</v>
+        <v>components_Cloud_storyPoints</v>
       </c>
       <c r="E41" s="68" t="e">
         <f>MATCH(D41, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25105,7 +25115,7 @@
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>StreamB</v>
+        <v>Dataverse</v>
       </c>
       <c r="B42" s="88" cm="1">
         <f t="array" ref="B42">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E42), 0)</f>
@@ -25113,7 +25123,7 @@
       </c>
       <c r="D42" s="68" t="str">
         <f t="shared" si="1"/>
-        <v>components_StreamB_storyPoints</v>
+        <v>components_Dataverse_storyPoints</v>
       </c>
       <c r="E42" s="68" t="e">
         <f>MATCH(D42, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25123,7 +25133,7 @@
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>StreamC</v>
+        <v>Architecture</v>
       </c>
       <c r="B43" s="88" cm="1">
         <f t="array" ref="B43">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E43), 0)</f>
@@ -25131,7 +25141,7 @@
       </c>
       <c r="D43" s="68" t="str">
         <f t="shared" si="1"/>
-        <v>components_StreamC_storyPoints</v>
+        <v>components_Architecture_storyPoints</v>
       </c>
       <c r="E43" s="68" t="e">
         <f>MATCH(D43, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25285,7 +25295,7 @@
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>StreamA</v>
+        <v>Cloud</v>
       </c>
       <c r="B53" s="88" cm="1">
         <f t="array" ref="B53">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E53), 0)</f>
@@ -25293,7 +25303,7 @@
       </c>
       <c r="D53" s="68" t="str">
         <f t="shared" ref="D53:D62" si="2">_xlfn.CONCAT("completedComponents_", A53,"_",D$15)</f>
-        <v>completedComponents_StreamA_storyPoints</v>
+        <v>completedComponents_Cloud_storyPoints</v>
       </c>
       <c r="E53" s="68" t="e">
         <f>MATCH(D53, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25303,7 +25313,7 @@
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>StreamB</v>
+        <v>Dataverse</v>
       </c>
       <c r="B54" s="88" cm="1">
         <f t="array" ref="B54">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E54), 0)</f>
@@ -25311,7 +25321,7 @@
       </c>
       <c r="D54" s="68" t="str">
         <f t="shared" si="2"/>
-        <v>completedComponents_StreamB_storyPoints</v>
+        <v>completedComponents_Dataverse_storyPoints</v>
       </c>
       <c r="E54" s="68" t="e">
         <f>MATCH(D54, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25321,7 +25331,7 @@
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>StreamC</v>
+        <v>Architecture</v>
       </c>
       <c r="B55" s="88" cm="1">
         <f t="array" ref="B55">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E55), 0)</f>
@@ -25329,7 +25339,7 @@
       </c>
       <c r="D55" s="68" t="str">
         <f t="shared" si="2"/>
-        <v>completedComponents_StreamC_storyPoints</v>
+        <v>completedComponents_Architecture_storyPoints</v>
       </c>
       <c r="E55" s="68" t="e">
         <f>MATCH(D55, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25544,7 +25554,7 @@
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Project1</v>
+        <v>Convergence</v>
       </c>
       <c r="B70" s="53" cm="1">
         <f t="array" ref="B70">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E70), 0)</f>
@@ -25552,7 +25562,7 @@
       </c>
       <c r="D70" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A70,"_",D$66)</f>
-        <v>labels_Project1_count</v>
+        <v>labels_Convergence_count</v>
       </c>
       <c r="E70" s="68" t="e">
         <f>MATCH(D70, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25562,7 +25572,7 @@
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project2</v>
+        <v>Project</v>
       </c>
       <c r="B71" s="53" cm="1">
         <f t="array" ref="B71">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E71), 0)</f>
@@ -25570,7 +25580,7 @@
       </c>
       <c r="D71" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A71, "_",D$66)</f>
-        <v>labels_Project2_count</v>
+        <v>labels_Project_count</v>
       </c>
       <c r="E71" s="68" t="e">
         <f>MATCH(D71, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25741,7 +25751,7 @@
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Project1</v>
+        <v>Convergence</v>
       </c>
       <c r="B82" s="53" cm="1">
         <f t="array" ref="B82">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E82), 0)</f>
@@ -25749,7 +25759,7 @@
       </c>
       <c r="D82" s="68" t="str">
         <f t="shared" si="3"/>
-        <v>completedLabels_Project1_count</v>
+        <v>completedLabels_Convergence_count</v>
       </c>
       <c r="E82" s="68" t="e">
         <f>MATCH(D82, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25759,7 +25769,7 @@
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project2</v>
+        <v>Project</v>
       </c>
       <c r="B83" s="53" cm="1">
         <f t="array" ref="B83">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E83), 0)</f>
@@ -25767,7 +25777,7 @@
       </c>
       <c r="D83" s="68" t="str">
         <f t="shared" si="3"/>
-        <v>completedLabels_Project2_count</v>
+        <v>completedLabels_Project_count</v>
       </c>
       <c r="E83" s="68" t="e">
         <f>MATCH(D83, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25902,7 +25912,7 @@
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>StreamA</v>
+        <v>Cloud</v>
       </c>
       <c r="B92" s="88" cm="1">
         <f t="array" ref="B92">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E92), 0)</f>
@@ -25910,7 +25920,7 @@
       </c>
       <c r="D92" s="68" t="str">
         <f t="shared" ref="D92:D101" si="4">_xlfn.CONCAT("components_", A92,"_",D$66)</f>
-        <v>components_StreamA_count</v>
+        <v>components_Cloud_count</v>
       </c>
       <c r="E92" s="68" t="e">
         <f>MATCH(D92, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25920,7 +25930,7 @@
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>StreamB</v>
+        <v>Dataverse</v>
       </c>
       <c r="B93" s="88" cm="1">
         <f t="array" ref="B93">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E93), 0)</f>
@@ -25928,7 +25938,7 @@
       </c>
       <c r="D93" s="68" t="str">
         <f t="shared" si="4"/>
-        <v>components_StreamB_count</v>
+        <v>components_Dataverse_count</v>
       </c>
       <c r="E93" s="68" t="e">
         <f>MATCH(D93, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25938,7 +25948,7 @@
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>StreamC</v>
+        <v>Architecture</v>
       </c>
       <c r="B94" s="88" cm="1">
         <f t="array" ref="B94">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E94), 0)</f>
@@ -25946,7 +25956,7 @@
       </c>
       <c r="D94" s="68" t="str">
         <f t="shared" si="4"/>
-        <v>components_StreamC_count</v>
+        <v>components_Architecture_count</v>
       </c>
       <c r="E94" s="68" t="e">
         <f>MATCH(D94, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -26100,7 +26110,7 @@
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>StreamA</v>
+        <v>Cloud</v>
       </c>
       <c r="B104" s="88" cm="1">
         <f t="array" ref="B104">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E104), 0)</f>
@@ -26108,7 +26118,7 @@
       </c>
       <c r="D104" s="68" t="str">
         <f t="shared" ref="D104:D113" si="5">_xlfn.CONCAT("completedComponents_", A104,"_",D$66)</f>
-        <v>completedComponents_StreamA_count</v>
+        <v>completedComponents_Cloud_count</v>
       </c>
       <c r="E104" s="68" t="e">
         <f>MATCH(D104, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -26118,7 +26128,7 @@
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>StreamB</v>
+        <v>Dataverse</v>
       </c>
       <c r="B105" s="88" cm="1">
         <f t="array" ref="B105">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E105), 0)</f>
@@ -26126,7 +26136,7 @@
       </c>
       <c r="D105" s="68" t="str">
         <f t="shared" si="5"/>
-        <v>completedComponents_StreamB_count</v>
+        <v>completedComponents_Dataverse_count</v>
       </c>
       <c r="E105" s="68" t="e">
         <f>MATCH(D105, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -26136,7 +26146,7 @@
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>StreamC</v>
+        <v>Architecture</v>
       </c>
       <c r="B106" s="88" cm="1">
         <f t="array" ref="B106">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E106), 0)</f>
@@ -26144,7 +26154,7 @@
       </c>
       <c r="D106" s="68" t="str">
         <f t="shared" si="5"/>
-        <v>completedComponents_StreamC_count</v>
+        <v>completedComponents_Architecture_count</v>
       </c>
       <c r="E106" s="68" t="e">
         <f>MATCH(D106, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -30240,12 +30250,192 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="C2:D2"/>
+  <dimension ref="A1:CL2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C2" s="110"/>
-      <c r="D2" s="110"/>
+    <row r="1" spans="1:90" x14ac:dyDescent="0.2">
+      <c r="A1" s="134"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
+      <c r="I1" s="134"/>
+      <c r="J1" s="134"/>
+      <c r="K1" s="134"/>
+      <c r="L1" s="134"/>
+      <c r="M1" s="134"/>
+      <c r="N1" s="134"/>
+      <c r="O1" s="134"/>
+      <c r="P1" s="134"/>
+      <c r="Q1" s="134"/>
+      <c r="R1" s="134"/>
+      <c r="S1" s="134"/>
+      <c r="T1" s="134"/>
+      <c r="U1" s="134"/>
+      <c r="V1" s="134"/>
+      <c r="W1" s="134"/>
+      <c r="X1" s="134"/>
+      <c r="Y1" s="134"/>
+      <c r="Z1" s="134"/>
+      <c r="AA1" s="134"/>
+      <c r="AB1" s="134"/>
+      <c r="AC1" s="134"/>
+      <c r="AD1" s="134"/>
+      <c r="AE1" s="134"/>
+      <c r="AF1" s="134"/>
+      <c r="AG1" s="134"/>
+      <c r="AH1" s="134"/>
+      <c r="AI1" s="134"/>
+      <c r="AJ1" s="134"/>
+      <c r="AK1" s="134"/>
+      <c r="AL1" s="134"/>
+      <c r="AM1" s="134"/>
+      <c r="AN1" s="134"/>
+      <c r="AO1" s="134"/>
+      <c r="AP1" s="134"/>
+      <c r="AQ1" s="134"/>
+      <c r="AR1" s="134"/>
+      <c r="AS1" s="134"/>
+      <c r="AT1" s="134"/>
+      <c r="AU1" s="134"/>
+      <c r="AV1" s="134"/>
+      <c r="AW1" s="134"/>
+      <c r="AX1" s="134"/>
+      <c r="AY1" s="134"/>
+      <c r="AZ1" s="134"/>
+      <c r="BA1" s="134"/>
+      <c r="BB1" s="134"/>
+      <c r="BC1" s="134"/>
+      <c r="BD1" s="134"/>
+      <c r="BE1" s="134"/>
+      <c r="BF1" s="134"/>
+      <c r="BG1" s="134"/>
+      <c r="BH1" s="134"/>
+      <c r="BI1" s="134"/>
+      <c r="BJ1" s="134"/>
+      <c r="BK1" s="134"/>
+      <c r="BL1" s="134"/>
+      <c r="BM1" s="134"/>
+      <c r="BN1" s="134"/>
+      <c r="BO1" s="134"/>
+      <c r="BP1" s="134"/>
+      <c r="BQ1" s="134"/>
+      <c r="BR1" s="134"/>
+      <c r="BS1" s="134"/>
+      <c r="BT1" s="134"/>
+      <c r="BU1" s="134"/>
+      <c r="BV1" s="134"/>
+      <c r="BW1" s="134"/>
+      <c r="BX1" s="134"/>
+      <c r="BY1" s="134"/>
+      <c r="BZ1" s="134"/>
+      <c r="CA1" s="134"/>
+      <c r="CB1" s="134"/>
+      <c r="CC1" s="134"/>
+      <c r="CD1" s="134"/>
+      <c r="CE1" s="134"/>
+      <c r="CF1" s="134"/>
+      <c r="CG1" s="134"/>
+      <c r="CH1" s="134"/>
+      <c r="CI1" s="134"/>
+      <c r="CJ1" s="134"/>
+      <c r="CK1" s="134"/>
+      <c r="CL1" s="134"/>
+    </row>
+    <row r="2" spans="1:90" x14ac:dyDescent="0.2">
+      <c r="A2" s="134"/>
+      <c r="B2" s="135"/>
+      <c r="C2" s="136"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="135"/>
+      <c r="F2" s="135"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="135"/>
+      <c r="I2" s="135"/>
+      <c r="J2" s="135"/>
+      <c r="K2" s="135"/>
+      <c r="L2" s="135"/>
+      <c r="M2" s="135"/>
+      <c r="N2" s="135"/>
+      <c r="O2" s="135"/>
+      <c r="P2" s="135"/>
+      <c r="Q2" s="135"/>
+      <c r="R2" s="135"/>
+      <c r="S2" s="135"/>
+      <c r="T2" s="135"/>
+      <c r="U2" s="135"/>
+      <c r="V2" s="135"/>
+      <c r="W2" s="135"/>
+      <c r="X2" s="135"/>
+      <c r="Y2" s="135"/>
+      <c r="Z2" s="135"/>
+      <c r="AA2" s="135"/>
+      <c r="AB2" s="135"/>
+      <c r="AC2" s="135"/>
+      <c r="AD2" s="135"/>
+      <c r="AE2" s="135"/>
+      <c r="AF2" s="135"/>
+      <c r="AG2" s="135"/>
+      <c r="AH2" s="135"/>
+      <c r="AI2" s="135"/>
+      <c r="AJ2" s="135"/>
+      <c r="AK2" s="135"/>
+      <c r="AL2" s="135"/>
+      <c r="AM2" s="135"/>
+      <c r="AN2" s="135"/>
+      <c r="AO2" s="135"/>
+      <c r="AP2" s="135"/>
+      <c r="AQ2" s="135"/>
+      <c r="AR2" s="135"/>
+      <c r="AS2" s="135"/>
+      <c r="AT2" s="135"/>
+      <c r="AU2" s="135"/>
+      <c r="AV2" s="135"/>
+      <c r="AW2" s="135"/>
+      <c r="AX2" s="135"/>
+      <c r="AY2" s="135"/>
+      <c r="AZ2" s="135"/>
+      <c r="BA2" s="135"/>
+      <c r="BB2" s="135"/>
+      <c r="BC2" s="135"/>
+      <c r="BD2" s="135"/>
+      <c r="BE2" s="135"/>
+      <c r="BF2" s="135"/>
+      <c r="BG2" s="135"/>
+      <c r="BH2" s="135"/>
+      <c r="BI2" s="135"/>
+      <c r="BJ2" s="135"/>
+      <c r="BK2" s="135"/>
+      <c r="BL2" s="135"/>
+      <c r="BM2" s="135"/>
+      <c r="BN2" s="135"/>
+      <c r="BO2" s="135"/>
+      <c r="BP2" s="135"/>
+      <c r="BQ2" s="135"/>
+      <c r="BR2" s="135"/>
+      <c r="BS2" s="135"/>
+      <c r="BT2" s="135"/>
+      <c r="BU2" s="135"/>
+      <c r="BV2" s="135"/>
+      <c r="BW2" s="135"/>
+      <c r="BX2" s="135"/>
+      <c r="BY2" s="135"/>
+      <c r="BZ2" s="135"/>
+      <c r="CA2" s="135"/>
+      <c r="CB2" s="135"/>
+      <c r="CC2" s="135"/>
+      <c r="CD2" s="135"/>
+      <c r="CE2" s="135"/>
+      <c r="CF2" s="135"/>
+      <c r="CG2" s="135"/>
+      <c r="CH2" s="135"/>
+      <c r="CI2" s="135"/>
+      <c r="CJ2" s="135"/>
+      <c r="CK2" s="135"/>
+      <c r="CL2" s="135"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix bug with excel workbook template labels & components examples
</commit_message>
<xml_diff>
--- a/assets/xlsx/visualise-metrics.xlsx
+++ b/assets/xlsx/visualise-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA97840B-3A3D-6A4C-BCFF-85C5F38583D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECFCF0C0-FB19-2948-8DB0-C47209AA0035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="158">
   <si>
     <t>Done</t>
   </si>
@@ -572,16 +572,19 @@
     <t>metricConfidence_totalUnestimatedWorkitems</t>
   </si>
   <si>
-    <t>Project</t>
+    <t>component1</t>
   </si>
   <si>
-    <t>Cloud</t>
+    <t>component2</t>
   </si>
   <si>
-    <t>Dataverse</t>
+    <t>component3</t>
   </si>
   <si>
-    <t>Architecture</t>
+    <t>label1</t>
+  </si>
+  <si>
+    <t>label2</t>
   </si>
 </sst>
 </file>
@@ -1441,6 +1444,9 @@
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1513,9 +1519,6 @@
     <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
@@ -1929,10 +1932,10 @@
                   <c:v>BAU/Improvement</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Convergence</c:v>
+                  <c:v>label1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Project</c:v>
+                  <c:v>label2</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3279,13 +3282,13 @@
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Cloud</c:v>
+                  <c:v>component1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Dataverse</c:v>
+                  <c:v>component2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Architecture</c:v>
+                  <c:v>component3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -8037,6 +8040,7 @@
               <a:latin typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
+            <a:pPr/>
             <a:t>0</a:t>
           </a:fld>
           <a:endParaRPr lang="en-AU" sz="3200" b="1">
@@ -13767,7 +13771,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>Convergence</a:t>
+                <a:t>label1</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -14096,7 +14100,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>Project</a:t>
+                <a:t>label2</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -15401,7 +15405,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>Cloud</a:t>
+                <a:t>component1</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -15730,7 +15734,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>Dataverse</a:t>
+                <a:t>component2</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -16056,7 +16060,7 @@
                   <a:cs typeface="Calibri"/>
                 </a:rPr>
                 <a:pPr algn="r"/>
-                <a:t>Architecture</a:t>
+                <a:t>component3</a:t>
               </a:fld>
               <a:endParaRPr lang="en-AU" sz="800">
                 <a:solidFill>
@@ -20199,30 +20203,30 @@
     </row>
     <row r="3" spans="2:13" ht="137" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="31"/>
-      <c r="C3" s="110"/>
-      <c r="D3" s="111"/>
-      <c r="E3" s="111"/>
-      <c r="F3" s="111"/>
-      <c r="G3" s="111"/>
-      <c r="H3" s="111"/>
-      <c r="I3" s="111"/>
-      <c r="J3" s="111"/>
-      <c r="K3" s="111"/>
-      <c r="L3" s="111"/>
+      <c r="C3" s="113"/>
+      <c r="D3" s="114"/>
+      <c r="E3" s="114"/>
+      <c r="F3" s="114"/>
+      <c r="G3" s="114"/>
+      <c r="H3" s="114"/>
+      <c r="I3" s="114"/>
+      <c r="J3" s="114"/>
+      <c r="K3" s="114"/>
+      <c r="L3" s="114"/>
       <c r="M3" s="36"/>
     </row>
     <row r="4" spans="2:13" ht="243.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="31"/>
       <c r="C4" s="29"/>
-      <c r="D4" s="117"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="124"/>
-      <c r="G4" s="124"/>
-      <c r="H4" s="124"/>
-      <c r="I4" s="125"/>
-      <c r="J4" s="123"/>
-      <c r="K4" s="124"/>
-      <c r="L4" s="125"/>
+      <c r="D4" s="120"/>
+      <c r="E4" s="121"/>
+      <c r="F4" s="127"/>
+      <c r="G4" s="127"/>
+      <c r="H4" s="127"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="126"/>
+      <c r="K4" s="127"/>
+      <c r="L4" s="128"/>
       <c r="M4" s="31"/>
     </row>
     <row r="5" spans="2:13" ht="226.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -20230,20 +20234,20 @@
       <c r="C5" s="30"/>
       <c r="D5" s="48"/>
       <c r="E5" s="49"/>
-      <c r="F5" s="112"/>
-      <c r="G5" s="113"/>
-      <c r="H5" s="113"/>
-      <c r="I5" s="114"/>
-      <c r="J5" s="112"/>
-      <c r="K5" s="113"/>
-      <c r="L5" s="114"/>
+      <c r="F5" s="115"/>
+      <c r="G5" s="116"/>
+      <c r="H5" s="116"/>
+      <c r="I5" s="117"/>
+      <c r="J5" s="115"/>
+      <c r="K5" s="116"/>
+      <c r="L5" s="117"/>
       <c r="M5" s="31"/>
     </row>
     <row r="6" spans="2:13" ht="26.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="31"/>
-      <c r="C6" s="115"/>
-      <c r="D6" s="119"/>
-      <c r="E6" s="120"/>
+      <c r="C6" s="118"/>
+      <c r="D6" s="122"/>
+      <c r="E6" s="123"/>
       <c r="F6" s="35"/>
       <c r="G6" s="37"/>
       <c r="H6" s="38"/>
@@ -20255,27 +20259,27 @@
     </row>
     <row r="7" spans="2:13" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="31"/>
-      <c r="C7" s="116"/>
-      <c r="D7" s="110"/>
-      <c r="E7" s="111"/>
+      <c r="C7" s="119"/>
+      <c r="D7" s="113"/>
+      <c r="E7" s="114"/>
       <c r="F7" s="34"/>
       <c r="G7" s="44"/>
-      <c r="H7" s="126" t="s">
+      <c r="H7" s="129" t="s">
         <v>60</v>
       </c>
-      <c r="I7" s="126"/>
-      <c r="J7" s="126" t="s">
+      <c r="I7" s="129"/>
+      <c r="J7" s="129" t="s">
         <v>61</v>
       </c>
-      <c r="K7" s="126"/>
+      <c r="K7" s="129"/>
       <c r="L7" s="40"/>
       <c r="M7" s="31"/>
     </row>
     <row r="8" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="31"/>
-      <c r="C8" s="116"/>
-      <c r="D8" s="110"/>
-      <c r="E8" s="111"/>
+      <c r="C8" s="119"/>
+      <c r="D8" s="113"/>
+      <c r="E8" s="114"/>
       <c r="F8" s="34"/>
       <c r="G8" s="46" t="s">
         <v>9</v>
@@ -20301,9 +20305,9 @@
     </row>
     <row r="9" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="31"/>
-      <c r="C9" s="116"/>
-      <c r="D9" s="110"/>
-      <c r="E9" s="111"/>
+      <c r="C9" s="119"/>
+      <c r="D9" s="113"/>
+      <c r="E9" s="114"/>
       <c r="F9" s="34"/>
       <c r="G9" s="50" t="s">
         <v>10</v>
@@ -20332,9 +20336,9 @@
     </row>
     <row r="10" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="31"/>
-      <c r="C10" s="116"/>
-      <c r="D10" s="110"/>
-      <c r="E10" s="111"/>
+      <c r="C10" s="119"/>
+      <c r="D10" s="113"/>
+      <c r="E10" s="114"/>
       <c r="F10" s="34"/>
       <c r="G10" s="51" t="s">
         <v>56</v>
@@ -20363,9 +20367,9 @@
     </row>
     <row r="11" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="31"/>
-      <c r="C11" s="116"/>
-      <c r="D11" s="110"/>
-      <c r="E11" s="111"/>
+      <c r="C11" s="119"/>
+      <c r="D11" s="113"/>
+      <c r="E11" s="114"/>
       <c r="F11" s="34"/>
       <c r="G11" s="46" t="s">
         <v>59</v>
@@ -20391,9 +20395,9 @@
     </row>
     <row r="12" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="31"/>
-      <c r="C12" s="116"/>
-      <c r="D12" s="110"/>
-      <c r="E12" s="111"/>
+      <c r="C12" s="119"/>
+      <c r="D12" s="113"/>
+      <c r="E12" s="114"/>
       <c r="F12" s="34"/>
       <c r="G12" s="46" t="s">
         <v>57</v>
@@ -20419,9 +20423,9 @@
     </row>
     <row r="13" spans="2:13" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="31"/>
-      <c r="C13" s="116"/>
-      <c r="D13" s="110"/>
-      <c r="E13" s="111"/>
+      <c r="C13" s="119"/>
+      <c r="D13" s="113"/>
+      <c r="E13" s="114"/>
       <c r="F13" s="34"/>
       <c r="G13" s="46" t="s">
         <v>58</v>
@@ -20447,9 +20451,9 @@
     </row>
     <row r="14" spans="2:13" ht="42.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B14" s="31"/>
-      <c r="C14" s="116"/>
-      <c r="D14" s="121"/>
-      <c r="E14" s="122"/>
+      <c r="C14" s="119"/>
+      <c r="D14" s="124"/>
+      <c r="E14" s="125"/>
       <c r="F14" s="33"/>
       <c r="G14" s="41"/>
       <c r="H14" s="42"/>
@@ -20461,16 +20465,16 @@
     </row>
     <row r="15" spans="2:13" ht="264.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B15" s="31"/>
-      <c r="C15" s="116"/>
-      <c r="D15" s="117"/>
-      <c r="E15" s="118"/>
-      <c r="F15" s="112"/>
-      <c r="G15" s="113"/>
-      <c r="H15" s="113"/>
-      <c r="I15" s="113"/>
-      <c r="J15" s="113"/>
-      <c r="K15" s="113"/>
-      <c r="L15" s="114"/>
+      <c r="C15" s="119"/>
+      <c r="D15" s="120"/>
+      <c r="E15" s="121"/>
+      <c r="F15" s="115"/>
+      <c r="G15" s="116"/>
+      <c r="H15" s="116"/>
+      <c r="I15" s="116"/>
+      <c r="J15" s="116"/>
+      <c r="K15" s="116"/>
+      <c r="L15" s="117"/>
       <c r="M15" s="36"/>
     </row>
     <row r="16" spans="2:13" ht="10" customHeight="1" x14ac:dyDescent="0.2">
@@ -21234,7 +21238,7 @@
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Convergence</v>
+        <v>label1</v>
       </c>
       <c r="B30" s="54">
         <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A30, 'Calculated Stats'!B$36:B$45, 0))</f>
@@ -21266,7 +21270,7 @@
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project</v>
+        <v>label2</v>
       </c>
       <c r="B31" s="54">
         <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A31, 'Calculated Stats'!B$36:B$45, 0))</f>
@@ -21411,7 +21415,7 @@
       <c r="O40" s="4"/>
       <c r="Q40" s="4" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>Cloud</v>
+        <v>component1</v>
       </c>
       <c r="R40" s="4">
         <f>INDEX('Calculated Stats'!D$66:D$75, MATCH(Q40, 'Calculated Stats'!B$66:B$75, 0))</f>
@@ -21440,7 +21444,7 @@
       <c r="O41" s="4"/>
       <c r="Q41" s="4" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>Dataverse</v>
+        <v>component2</v>
       </c>
       <c r="R41" s="4">
         <f>INDEX('Calculated Stats'!D$66:D$75, MATCH(Q41, 'Calculated Stats'!B$66:B$75, 0))</f>
@@ -21465,7 +21469,7 @@
       <c r="O42" s="4"/>
       <c r="Q42" s="4" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>Architecture</v>
+        <v>component3</v>
       </c>
       <c r="R42" s="4">
         <f>INDEX('Calculated Stats'!D$66:D$75, MATCH(Q42, 'Calculated Stats'!B$66:B$75, 0))</f>
@@ -21917,10 +21921,10 @@
       <c r="G5" s="105"/>
     </row>
     <row r="6" spans="2:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="127" t="s">
+      <c r="B6" s="130" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="128"/>
+      <c r="C6" s="131"/>
       <c r="D6" s="105"/>
       <c r="E6" s="105"/>
       <c r="F6" s="106"/>
@@ -21943,7 +21947,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="79" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D8" s="105"/>
       <c r="E8" s="105"/>
@@ -21955,7 +21959,7 @@
         <v>53</v>
       </c>
       <c r="C9" s="79" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D9" s="105"/>
       <c r="E9" s="105"/>
@@ -21964,10 +21968,10 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="76" t="s">
-        <v>2</v>
+        <v>156</v>
       </c>
       <c r="C10" s="79" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D10" s="105"/>
       <c r="E10" s="105"/>
@@ -21976,7 +21980,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="76" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C11" s="79"/>
       <c r="D11" s="105"/>
@@ -22191,10 +22195,10 @@
       <c r="G31" s="105"/>
     </row>
     <row r="32" spans="2:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="127" t="s">
+      <c r="B32" s="130" t="s">
         <v>135</v>
       </c>
-      <c r="C32" s="128"/>
+      <c r="C32" s="131"/>
       <c r="D32" s="28"/>
       <c r="E32" s="28"/>
       <c r="F32" s="94"/>
@@ -22213,10 +22217,10 @@
       <c r="B34" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C34" s="132" t="s">
+      <c r="C34" s="135" t="s">
         <v>5</v>
       </c>
-      <c r="D34" s="132"/>
+      <c r="D34" s="135"/>
       <c r="E34" s="105"/>
       <c r="F34" s="105"/>
       <c r="G34" s="104"/>
@@ -22276,7 +22280,7 @@
     <row r="38" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B38" s="82" t="str">
         <f t="shared" si="0"/>
-        <v>Convergence</v>
+        <v>label1</v>
       </c>
       <c r="C38" s="4">
         <f>'processed | data'!B19</f>
@@ -22294,7 +22298,7 @@
     <row r="39" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B39" s="82" t="str">
         <f t="shared" si="0"/>
-        <v>Project</v>
+        <v>label2</v>
       </c>
       <c r="C39" s="4">
         <f>'processed | data'!B20</f>
@@ -22448,10 +22452,10 @@
       <c r="B49" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C49" s="132" t="s">
+      <c r="C49" s="135" t="s">
         <v>83</v>
       </c>
-      <c r="D49" s="132"/>
+      <c r="D49" s="135"/>
       <c r="E49" s="105"/>
       <c r="F49" s="105"/>
       <c r="G49" s="105"/>
@@ -22511,7 +22515,7 @@
     <row r="53" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B53" s="82" t="str">
         <f t="shared" si="1"/>
-        <v>Convergence</v>
+        <v>label1</v>
       </c>
       <c r="C53" s="4">
         <f>'processed | data'!B70</f>
@@ -22529,7 +22533,7 @@
     <row r="54" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B54" s="82" t="str">
         <f t="shared" si="1"/>
-        <v>Project</v>
+        <v>label2</v>
       </c>
       <c r="C54" s="4">
         <f>'processed | data'!B71</f>
@@ -22683,10 +22687,10 @@
       <c r="B64" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C64" s="133" t="s">
+      <c r="C64" s="136" t="s">
         <v>5</v>
       </c>
-      <c r="D64" s="133"/>
+      <c r="D64" s="136"/>
       <c r="E64" s="105"/>
       <c r="F64" s="105"/>
       <c r="G64" s="105"/>
@@ -22710,7 +22714,7 @@
     <row r="66" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B66" s="82" t="str">
         <f>C8</f>
-        <v>Cloud</v>
+        <v>component1</v>
       </c>
       <c r="C66" s="101">
         <f>'processed | data'!B41</f>
@@ -22728,7 +22732,7 @@
     <row r="67" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B67" s="82" t="str">
         <f t="shared" ref="B67:B75" si="2">C9</f>
-        <v>Dataverse</v>
+        <v>component2</v>
       </c>
       <c r="C67" s="101">
         <f>'processed | data'!B42</f>
@@ -22746,7 +22750,7 @@
     <row r="68" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B68" s="82" t="str">
         <f t="shared" si="2"/>
-        <v>Architecture</v>
+        <v>component3</v>
       </c>
       <c r="C68" s="101">
         <f>'processed | data'!B43</f>
@@ -22918,10 +22922,10 @@
       <c r="B79" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="C79" s="133" t="s">
+      <c r="C79" s="136" t="s">
         <v>83</v>
       </c>
-      <c r="D79" s="133"/>
+      <c r="D79" s="136"/>
       <c r="E79" s="105"/>
       <c r="F79" s="105"/>
       <c r="G79" s="105"/>
@@ -22945,7 +22949,7 @@
     <row r="81" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B81" s="82" t="str">
         <f>C8</f>
-        <v>Cloud</v>
+        <v>component1</v>
       </c>
       <c r="C81" s="101">
         <f>'processed | data'!B92</f>
@@ -22963,7 +22967,7 @@
     <row r="82" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B82" s="82" t="str">
         <f t="shared" ref="B82:B90" si="3">C9</f>
-        <v>Dataverse</v>
+        <v>component2</v>
       </c>
       <c r="C82" s="101">
         <f>'processed | data'!B93</f>
@@ -22981,7 +22985,7 @@
     <row r="83" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B83" s="82" t="str">
         <f t="shared" si="3"/>
-        <v>Architecture</v>
+        <v>component3</v>
       </c>
       <c r="C83" s="101">
         <f>'processed | data'!B94</f>
@@ -23304,14 +23308,14 @@
     </row>
     <row r="104" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B104" s="6"/>
-      <c r="C104" s="129" t="s">
+      <c r="C104" s="132" t="s">
         <v>6</v>
       </c>
-      <c r="D104" s="130"/>
-      <c r="E104" s="129" t="s">
+      <c r="D104" s="133"/>
+      <c r="E104" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="F104" s="131"/>
+      <c r="F104" s="134"/>
       <c r="G104" s="6"/>
       <c r="N104" s="107"/>
     </row>
@@ -24739,7 +24743,7 @@
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Convergence</v>
+        <v>label1</v>
       </c>
       <c r="B19" s="53" cm="1">
         <f t="array" ref="B19">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E19), 0)</f>
@@ -24747,7 +24751,7 @@
       </c>
       <c r="D19" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A19,"_",D$15)</f>
-        <v>labels_Convergence_storyPoints</v>
+        <v>labels_label1_storyPoints</v>
       </c>
       <c r="E19" s="68" t="e">
         <f>MATCH(D19, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -24757,7 +24761,7 @@
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project</v>
+        <v>label2</v>
       </c>
       <c r="B20" s="53" cm="1">
         <f t="array" ref="B20">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E20), 0)</f>
@@ -24765,7 +24769,7 @@
       </c>
       <c r="D20" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A20, "_",D$15)</f>
-        <v>labels_Project_storyPoints</v>
+        <v>labels_label2_storyPoints</v>
       </c>
       <c r="E20" s="68" t="e">
         <f>MATCH(D20, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -24936,7 +24940,7 @@
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Convergence</v>
+        <v>label1</v>
       </c>
       <c r="B31" s="53" cm="1">
         <f t="array" ref="B31">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E31), 0)</f>
@@ -24944,7 +24948,7 @@
       </c>
       <c r="D31" s="68" t="str">
         <f t="shared" si="0"/>
-        <v>completedLabels_Convergence_storyPoints</v>
+        <v>completedLabels_label1_storyPoints</v>
       </c>
       <c r="E31" s="68" t="e">
         <f>MATCH(D31, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -24954,7 +24958,7 @@
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project</v>
+        <v>label2</v>
       </c>
       <c r="B32" s="53" cm="1">
         <f t="array" ref="B32">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E32), 0)</f>
@@ -24962,7 +24966,7 @@
       </c>
       <c r="D32" s="68" t="str">
         <f t="shared" si="0"/>
-        <v>completedLabels_Project_storyPoints</v>
+        <v>completedLabels_label2_storyPoints</v>
       </c>
       <c r="E32" s="68" t="e">
         <f>MATCH(D32, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25097,7 +25101,7 @@
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>Cloud</v>
+        <v>component1</v>
       </c>
       <c r="B41" s="88" cm="1">
         <f t="array" ref="B41">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E41), 0)</f>
@@ -25105,7 +25109,7 @@
       </c>
       <c r="D41" s="68" t="str">
         <f t="shared" ref="D41:D50" si="1">_xlfn.CONCAT("components_", A41,"_",D$15)</f>
-        <v>components_Cloud_storyPoints</v>
+        <v>components_component1_storyPoints</v>
       </c>
       <c r="E41" s="68" t="e">
         <f>MATCH(D41, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25115,7 +25119,7 @@
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>Dataverse</v>
+        <v>component2</v>
       </c>
       <c r="B42" s="88" cm="1">
         <f t="array" ref="B42">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E42), 0)</f>
@@ -25123,7 +25127,7 @@
       </c>
       <c r="D42" s="68" t="str">
         <f t="shared" si="1"/>
-        <v>components_Dataverse_storyPoints</v>
+        <v>components_component2_storyPoints</v>
       </c>
       <c r="E42" s="68" t="e">
         <f>MATCH(D42, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25133,7 +25137,7 @@
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>Architecture</v>
+        <v>component3</v>
       </c>
       <c r="B43" s="88" cm="1">
         <f t="array" ref="B43">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E43), 0)</f>
@@ -25141,7 +25145,7 @@
       </c>
       <c r="D43" s="68" t="str">
         <f t="shared" si="1"/>
-        <v>components_Architecture_storyPoints</v>
+        <v>components_component3_storyPoints</v>
       </c>
       <c r="E43" s="68" t="e">
         <f>MATCH(D43, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25295,7 +25299,7 @@
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>Cloud</v>
+        <v>component1</v>
       </c>
       <c r="B53" s="88" cm="1">
         <f t="array" ref="B53">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E53), 0)</f>
@@ -25303,7 +25307,7 @@
       </c>
       <c r="D53" s="68" t="str">
         <f t="shared" ref="D53:D62" si="2">_xlfn.CONCAT("completedComponents_", A53,"_",D$15)</f>
-        <v>completedComponents_Cloud_storyPoints</v>
+        <v>completedComponents_component1_storyPoints</v>
       </c>
       <c r="E53" s="68" t="e">
         <f>MATCH(D53, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25313,7 +25317,7 @@
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>Dataverse</v>
+        <v>component2</v>
       </c>
       <c r="B54" s="88" cm="1">
         <f t="array" ref="B54">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E54), 0)</f>
@@ -25321,7 +25325,7 @@
       </c>
       <c r="D54" s="68" t="str">
         <f t="shared" si="2"/>
-        <v>completedComponents_Dataverse_storyPoints</v>
+        <v>completedComponents_component2_storyPoints</v>
       </c>
       <c r="E54" s="68" t="e">
         <f>MATCH(D54, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25331,7 +25335,7 @@
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>Architecture</v>
+        <v>component3</v>
       </c>
       <c r="B55" s="88" cm="1">
         <f t="array" ref="B55">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E55), 0)</f>
@@ -25339,7 +25343,7 @@
       </c>
       <c r="D55" s="68" t="str">
         <f t="shared" si="2"/>
-        <v>completedComponents_Architecture_storyPoints</v>
+        <v>completedComponents_component3_storyPoints</v>
       </c>
       <c r="E55" s="68" t="e">
         <f>MATCH(D55, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25554,7 +25558,7 @@
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Convergence</v>
+        <v>label1</v>
       </c>
       <c r="B70" s="53" cm="1">
         <f t="array" ref="B70">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E70), 0)</f>
@@ -25562,7 +25566,7 @@
       </c>
       <c r="D70" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A70,"_",D$66)</f>
-        <v>labels_Convergence_count</v>
+        <v>labels_label1_count</v>
       </c>
       <c r="E70" s="68" t="e">
         <f>MATCH(D70, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25572,7 +25576,7 @@
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project</v>
+        <v>label2</v>
       </c>
       <c r="B71" s="53" cm="1">
         <f t="array" ref="B71">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E71), 0)</f>
@@ -25580,7 +25584,7 @@
       </c>
       <c r="D71" s="68" t="str">
         <f>_xlfn.CONCAT("labels_", A71, "_",D$66)</f>
-        <v>labels_Project_count</v>
+        <v>labels_label2_count</v>
       </c>
       <c r="E71" s="68" t="e">
         <f>MATCH(D71, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25751,7 +25755,7 @@
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="84" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>Convergence</v>
+        <v>label1</v>
       </c>
       <c r="B82" s="53" cm="1">
         <f t="array" ref="B82">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E82), 0)</f>
@@ -25759,7 +25763,7 @@
       </c>
       <c r="D82" s="68" t="str">
         <f t="shared" si="3"/>
-        <v>completedLabels_Convergence_count</v>
+        <v>completedLabels_label1_count</v>
       </c>
       <c r="E82" s="68" t="e">
         <f>MATCH(D82, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25769,7 +25773,7 @@
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="84" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>Project</v>
+        <v>label2</v>
       </c>
       <c r="B83" s="53" cm="1">
         <f t="array" ref="B83">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E83), 0)</f>
@@ -25777,7 +25781,7 @@
       </c>
       <c r="D83" s="68" t="str">
         <f t="shared" si="3"/>
-        <v>completedLabels_Project_count</v>
+        <v>completedLabels_label2_count</v>
       </c>
       <c r="E83" s="68" t="e">
         <f>MATCH(D83, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25912,7 +25916,7 @@
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>Cloud</v>
+        <v>component1</v>
       </c>
       <c r="B92" s="88" cm="1">
         <f t="array" ref="B92">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E92), 0)</f>
@@ -25920,7 +25924,7 @@
       </c>
       <c r="D92" s="68" t="str">
         <f t="shared" ref="D92:D101" si="4">_xlfn.CONCAT("components_", A92,"_",D$66)</f>
-        <v>components_Cloud_count</v>
+        <v>components_component1_count</v>
       </c>
       <c r="E92" s="68" t="e">
         <f>MATCH(D92, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25930,7 +25934,7 @@
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>Dataverse</v>
+        <v>component2</v>
       </c>
       <c r="B93" s="88" cm="1">
         <f t="array" ref="B93">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E93), 0)</f>
@@ -25938,7 +25942,7 @@
       </c>
       <c r="D93" s="68" t="str">
         <f t="shared" si="4"/>
-        <v>components_Dataverse_count</v>
+        <v>components_component2_count</v>
       </c>
       <c r="E93" s="68" t="e">
         <f>MATCH(D93, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -25948,7 +25952,7 @@
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>Architecture</v>
+        <v>component3</v>
       </c>
       <c r="B94" s="88" cm="1">
         <f t="array" ref="B94">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E94), 0)</f>
@@ -25956,7 +25960,7 @@
       </c>
       <c r="D94" s="68" t="str">
         <f t="shared" si="4"/>
-        <v>components_Architecture_count</v>
+        <v>components_component3_count</v>
       </c>
       <c r="E94" s="68" t="e">
         <f>MATCH(D94, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -26110,7 +26114,7 @@
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" s="87" t="str">
         <f>'Calculated Stats'!C8</f>
-        <v>Cloud</v>
+        <v>component1</v>
       </c>
       <c r="B104" s="88" cm="1">
         <f t="array" ref="B104">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E104), 0)</f>
@@ -26118,7 +26122,7 @@
       </c>
       <c r="D104" s="68" t="str">
         <f t="shared" ref="D104:D113" si="5">_xlfn.CONCAT("completedComponents_", A104,"_",D$66)</f>
-        <v>completedComponents_Cloud_count</v>
+        <v>completedComponents_component1_count</v>
       </c>
       <c r="E104" s="68" t="e">
         <f>MATCH(D104, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -26128,7 +26132,7 @@
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" s="87" t="str">
         <f>'Calculated Stats'!C9</f>
-        <v>Dataverse</v>
+        <v>component2</v>
       </c>
       <c r="B105" s="88" cm="1">
         <f t="array" ref="B105">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E105), 0)</f>
@@ -26136,7 +26140,7 @@
       </c>
       <c r="D105" s="68" t="str">
         <f t="shared" si="5"/>
-        <v>completedComponents_Dataverse_count</v>
+        <v>completedComponents_component2_count</v>
       </c>
       <c r="E105" s="68" t="e">
         <f>MATCH(D105, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -26146,7 +26150,7 @@
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" s="87" t="str">
         <f>'Calculated Stats'!C10</f>
-        <v>Architecture</v>
+        <v>component3</v>
       </c>
       <c r="B106" s="88" cm="1">
         <f t="array" ref="B106">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E106), 0)</f>
@@ -26154,7 +26158,7 @@
       </c>
       <c r="D106" s="68" t="str">
         <f t="shared" si="5"/>
-        <v>completedComponents_Architecture_count</v>
+        <v>completedComponents_component3_count</v>
       </c>
       <c r="E106" s="68" t="e">
         <f>MATCH(D106, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -30254,188 +30258,188 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:90" x14ac:dyDescent="0.2">
-      <c r="A1" s="134"/>
-      <c r="B1" s="134"/>
-      <c r="C1" s="134"/>
-      <c r="D1" s="134"/>
-      <c r="E1" s="134"/>
-      <c r="F1" s="134"/>
-      <c r="G1" s="134"/>
-      <c r="H1" s="134"/>
-      <c r="I1" s="134"/>
-      <c r="J1" s="134"/>
-      <c r="K1" s="134"/>
-      <c r="L1" s="134"/>
-      <c r="M1" s="134"/>
-      <c r="N1" s="134"/>
-      <c r="O1" s="134"/>
-      <c r="P1" s="134"/>
-      <c r="Q1" s="134"/>
-      <c r="R1" s="134"/>
-      <c r="S1" s="134"/>
-      <c r="T1" s="134"/>
-      <c r="U1" s="134"/>
-      <c r="V1" s="134"/>
-      <c r="W1" s="134"/>
-      <c r="X1" s="134"/>
-      <c r="Y1" s="134"/>
-      <c r="Z1" s="134"/>
-      <c r="AA1" s="134"/>
-      <c r="AB1" s="134"/>
-      <c r="AC1" s="134"/>
-      <c r="AD1" s="134"/>
-      <c r="AE1" s="134"/>
-      <c r="AF1" s="134"/>
-      <c r="AG1" s="134"/>
-      <c r="AH1" s="134"/>
-      <c r="AI1" s="134"/>
-      <c r="AJ1" s="134"/>
-      <c r="AK1" s="134"/>
-      <c r="AL1" s="134"/>
-      <c r="AM1" s="134"/>
-      <c r="AN1" s="134"/>
-      <c r="AO1" s="134"/>
-      <c r="AP1" s="134"/>
-      <c r="AQ1" s="134"/>
-      <c r="AR1" s="134"/>
-      <c r="AS1" s="134"/>
-      <c r="AT1" s="134"/>
-      <c r="AU1" s="134"/>
-      <c r="AV1" s="134"/>
-      <c r="AW1" s="134"/>
-      <c r="AX1" s="134"/>
-      <c r="AY1" s="134"/>
-      <c r="AZ1" s="134"/>
-      <c r="BA1" s="134"/>
-      <c r="BB1" s="134"/>
-      <c r="BC1" s="134"/>
-      <c r="BD1" s="134"/>
-      <c r="BE1" s="134"/>
-      <c r="BF1" s="134"/>
-      <c r="BG1" s="134"/>
-      <c r="BH1" s="134"/>
-      <c r="BI1" s="134"/>
-      <c r="BJ1" s="134"/>
-      <c r="BK1" s="134"/>
-      <c r="BL1" s="134"/>
-      <c r="BM1" s="134"/>
-      <c r="BN1" s="134"/>
-      <c r="BO1" s="134"/>
-      <c r="BP1" s="134"/>
-      <c r="BQ1" s="134"/>
-      <c r="BR1" s="134"/>
-      <c r="BS1" s="134"/>
-      <c r="BT1" s="134"/>
-      <c r="BU1" s="134"/>
-      <c r="BV1" s="134"/>
-      <c r="BW1" s="134"/>
-      <c r="BX1" s="134"/>
-      <c r="BY1" s="134"/>
-      <c r="BZ1" s="134"/>
-      <c r="CA1" s="134"/>
-      <c r="CB1" s="134"/>
-      <c r="CC1" s="134"/>
-      <c r="CD1" s="134"/>
-      <c r="CE1" s="134"/>
-      <c r="CF1" s="134"/>
-      <c r="CG1" s="134"/>
-      <c r="CH1" s="134"/>
-      <c r="CI1" s="134"/>
-      <c r="CJ1" s="134"/>
-      <c r="CK1" s="134"/>
-      <c r="CL1" s="134"/>
+      <c r="A1" s="110"/>
+      <c r="B1" s="110"/>
+      <c r="C1" s="110"/>
+      <c r="D1" s="110"/>
+      <c r="E1" s="110"/>
+      <c r="F1" s="110"/>
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="110"/>
+      <c r="P1" s="110"/>
+      <c r="Q1" s="110"/>
+      <c r="R1" s="110"/>
+      <c r="S1" s="110"/>
+      <c r="T1" s="110"/>
+      <c r="U1" s="110"/>
+      <c r="V1" s="110"/>
+      <c r="W1" s="110"/>
+      <c r="X1" s="110"/>
+      <c r="Y1" s="110"/>
+      <c r="Z1" s="110"/>
+      <c r="AA1" s="110"/>
+      <c r="AB1" s="110"/>
+      <c r="AC1" s="110"/>
+      <c r="AD1" s="110"/>
+      <c r="AE1" s="110"/>
+      <c r="AF1" s="110"/>
+      <c r="AG1" s="110"/>
+      <c r="AH1" s="110"/>
+      <c r="AI1" s="110"/>
+      <c r="AJ1" s="110"/>
+      <c r="AK1" s="110"/>
+      <c r="AL1" s="110"/>
+      <c r="AM1" s="110"/>
+      <c r="AN1" s="110"/>
+      <c r="AO1" s="110"/>
+      <c r="AP1" s="110"/>
+      <c r="AQ1" s="110"/>
+      <c r="AR1" s="110"/>
+      <c r="AS1" s="110"/>
+      <c r="AT1" s="110"/>
+      <c r="AU1" s="110"/>
+      <c r="AV1" s="110"/>
+      <c r="AW1" s="110"/>
+      <c r="AX1" s="110"/>
+      <c r="AY1" s="110"/>
+      <c r="AZ1" s="110"/>
+      <c r="BA1" s="110"/>
+      <c r="BB1" s="110"/>
+      <c r="BC1" s="110"/>
+      <c r="BD1" s="110"/>
+      <c r="BE1" s="110"/>
+      <c r="BF1" s="110"/>
+      <c r="BG1" s="110"/>
+      <c r="BH1" s="110"/>
+      <c r="BI1" s="110"/>
+      <c r="BJ1" s="110"/>
+      <c r="BK1" s="110"/>
+      <c r="BL1" s="110"/>
+      <c r="BM1" s="110"/>
+      <c r="BN1" s="110"/>
+      <c r="BO1" s="110"/>
+      <c r="BP1" s="110"/>
+      <c r="BQ1" s="110"/>
+      <c r="BR1" s="110"/>
+      <c r="BS1" s="110"/>
+      <c r="BT1" s="110"/>
+      <c r="BU1" s="110"/>
+      <c r="BV1" s="110"/>
+      <c r="BW1" s="110"/>
+      <c r="BX1" s="110"/>
+      <c r="BY1" s="110"/>
+      <c r="BZ1" s="110"/>
+      <c r="CA1" s="110"/>
+      <c r="CB1" s="110"/>
+      <c r="CC1" s="110"/>
+      <c r="CD1" s="110"/>
+      <c r="CE1" s="110"/>
+      <c r="CF1" s="110"/>
+      <c r="CG1" s="110"/>
+      <c r="CH1" s="110"/>
+      <c r="CI1" s="110"/>
+      <c r="CJ1" s="110"/>
+      <c r="CK1" s="110"/>
+      <c r="CL1" s="110"/>
     </row>
     <row r="2" spans="1:90" x14ac:dyDescent="0.2">
-      <c r="A2" s="134"/>
-      <c r="B2" s="135"/>
-      <c r="C2" s="136"/>
-      <c r="D2" s="136"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
-      <c r="I2" s="135"/>
-      <c r="J2" s="135"/>
-      <c r="K2" s="135"/>
-      <c r="L2" s="135"/>
-      <c r="M2" s="135"/>
-      <c r="N2" s="135"/>
-      <c r="O2" s="135"/>
-      <c r="P2" s="135"/>
-      <c r="Q2" s="135"/>
-      <c r="R2" s="135"/>
-      <c r="S2" s="135"/>
-      <c r="T2" s="135"/>
-      <c r="U2" s="135"/>
-      <c r="V2" s="135"/>
-      <c r="W2" s="135"/>
-      <c r="X2" s="135"/>
-      <c r="Y2" s="135"/>
-      <c r="Z2" s="135"/>
-      <c r="AA2" s="135"/>
-      <c r="AB2" s="135"/>
-      <c r="AC2" s="135"/>
-      <c r="AD2" s="135"/>
-      <c r="AE2" s="135"/>
-      <c r="AF2" s="135"/>
-      <c r="AG2" s="135"/>
-      <c r="AH2" s="135"/>
-      <c r="AI2" s="135"/>
-      <c r="AJ2" s="135"/>
-      <c r="AK2" s="135"/>
-      <c r="AL2" s="135"/>
-      <c r="AM2" s="135"/>
-      <c r="AN2" s="135"/>
-      <c r="AO2" s="135"/>
-      <c r="AP2" s="135"/>
-      <c r="AQ2" s="135"/>
-      <c r="AR2" s="135"/>
-      <c r="AS2" s="135"/>
-      <c r="AT2" s="135"/>
-      <c r="AU2" s="135"/>
-      <c r="AV2" s="135"/>
-      <c r="AW2" s="135"/>
-      <c r="AX2" s="135"/>
-      <c r="AY2" s="135"/>
-      <c r="AZ2" s="135"/>
-      <c r="BA2" s="135"/>
-      <c r="BB2" s="135"/>
-      <c r="BC2" s="135"/>
-      <c r="BD2" s="135"/>
-      <c r="BE2" s="135"/>
-      <c r="BF2" s="135"/>
-      <c r="BG2" s="135"/>
-      <c r="BH2" s="135"/>
-      <c r="BI2" s="135"/>
-      <c r="BJ2" s="135"/>
-      <c r="BK2" s="135"/>
-      <c r="BL2" s="135"/>
-      <c r="BM2" s="135"/>
-      <c r="BN2" s="135"/>
-      <c r="BO2" s="135"/>
-      <c r="BP2" s="135"/>
-      <c r="BQ2" s="135"/>
-      <c r="BR2" s="135"/>
-      <c r="BS2" s="135"/>
-      <c r="BT2" s="135"/>
-      <c r="BU2" s="135"/>
-      <c r="BV2" s="135"/>
-      <c r="BW2" s="135"/>
-      <c r="BX2" s="135"/>
-      <c r="BY2" s="135"/>
-      <c r="BZ2" s="135"/>
-      <c r="CA2" s="135"/>
-      <c r="CB2" s="135"/>
-      <c r="CC2" s="135"/>
-      <c r="CD2" s="135"/>
-      <c r="CE2" s="135"/>
-      <c r="CF2" s="135"/>
-      <c r="CG2" s="135"/>
-      <c r="CH2" s="135"/>
-      <c r="CI2" s="135"/>
-      <c r="CJ2" s="135"/>
-      <c r="CK2" s="135"/>
-      <c r="CL2" s="135"/>
+      <c r="A2" s="110"/>
+      <c r="B2" s="111"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="111"/>
+      <c r="P2" s="111"/>
+      <c r="Q2" s="111"/>
+      <c r="R2" s="111"/>
+      <c r="S2" s="111"/>
+      <c r="T2" s="111"/>
+      <c r="U2" s="111"/>
+      <c r="V2" s="111"/>
+      <c r="W2" s="111"/>
+      <c r="X2" s="111"/>
+      <c r="Y2" s="111"/>
+      <c r="Z2" s="111"/>
+      <c r="AA2" s="111"/>
+      <c r="AB2" s="111"/>
+      <c r="AC2" s="111"/>
+      <c r="AD2" s="111"/>
+      <c r="AE2" s="111"/>
+      <c r="AF2" s="111"/>
+      <c r="AG2" s="111"/>
+      <c r="AH2" s="111"/>
+      <c r="AI2" s="111"/>
+      <c r="AJ2" s="111"/>
+      <c r="AK2" s="111"/>
+      <c r="AL2" s="111"/>
+      <c r="AM2" s="111"/>
+      <c r="AN2" s="111"/>
+      <c r="AO2" s="111"/>
+      <c r="AP2" s="111"/>
+      <c r="AQ2" s="111"/>
+      <c r="AR2" s="111"/>
+      <c r="AS2" s="111"/>
+      <c r="AT2" s="111"/>
+      <c r="AU2" s="111"/>
+      <c r="AV2" s="111"/>
+      <c r="AW2" s="111"/>
+      <c r="AX2" s="111"/>
+      <c r="AY2" s="111"/>
+      <c r="AZ2" s="111"/>
+      <c r="BA2" s="111"/>
+      <c r="BB2" s="111"/>
+      <c r="BC2" s="111"/>
+      <c r="BD2" s="111"/>
+      <c r="BE2" s="111"/>
+      <c r="BF2" s="111"/>
+      <c r="BG2" s="111"/>
+      <c r="BH2" s="111"/>
+      <c r="BI2" s="111"/>
+      <c r="BJ2" s="111"/>
+      <c r="BK2" s="111"/>
+      <c r="BL2" s="111"/>
+      <c r="BM2" s="111"/>
+      <c r="BN2" s="111"/>
+      <c r="BO2" s="111"/>
+      <c r="BP2" s="111"/>
+      <c r="BQ2" s="111"/>
+      <c r="BR2" s="111"/>
+      <c r="BS2" s="111"/>
+      <c r="BT2" s="111"/>
+      <c r="BU2" s="111"/>
+      <c r="BV2" s="111"/>
+      <c r="BW2" s="111"/>
+      <c r="BX2" s="111"/>
+      <c r="BY2" s="111"/>
+      <c r="BZ2" s="111"/>
+      <c r="CA2" s="111"/>
+      <c r="CB2" s="111"/>
+      <c r="CC2" s="111"/>
+      <c r="CD2" s="111"/>
+      <c r="CE2" s="111"/>
+      <c r="CF2" s="111"/>
+      <c r="CG2" s="111"/>
+      <c r="CH2" s="111"/>
+      <c r="CI2" s="111"/>
+      <c r="CJ2" s="111"/>
+      <c r="CK2" s="111"/>
+      <c r="CL2" s="111"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Improve excel workbook template sample images
</commit_message>
<xml_diff>
--- a/assets/xlsx/visualise-metrics.xlsx
+++ b/assets/xlsx/visualise-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECFCF0C0-FB19-2948-8DB0-C47209AA0035}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E85F4774-714E-AF4E-B6E4-92F1BEFE9D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8243,7 +8243,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="889898" y="2482769"/>
+          <a:off x="878803" y="2466919"/>
           <a:ext cx="2470148" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
@@ -8407,7 +8407,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="864498" y="5579533"/>
+          <a:off x="853403" y="5560802"/>
           <a:ext cx="2676522" cy="530225"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2679967" cy="536575"/>
@@ -8609,8 +8609,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="861322" y="8451525"/>
-          <a:ext cx="3241673" cy="751930"/>
+          <a:off x="850227" y="8433082"/>
+          <a:ext cx="3241673" cy="758702"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3238163" cy="433685"/>
         </a:xfrm>
@@ -9007,7 +9007,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7963472" y="2492294"/>
+          <a:off x="7956412" y="2476444"/>
           <a:ext cx="2466973" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
@@ -9175,7 +9175,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7979347" y="5598583"/>
+          <a:off x="7972287" y="5579852"/>
           <a:ext cx="2355848" cy="530225"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2340804" cy="536575"/>
@@ -9322,7 +9322,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8079835" y="6160558"/>
+          <a:off x="8072775" y="6141827"/>
           <a:ext cx="2179786" cy="901700"/>
           <a:chOff x="6190137" y="5534025"/>
           <a:chExt cx="2182604" cy="901700"/>
@@ -9730,7 +9730,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10789385" y="5576358"/>
+          <a:off x="10780307" y="5557627"/>
           <a:ext cx="2403472" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2394604" cy="536575"/>
@@ -9960,8 +9960,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8020621" y="8480100"/>
-          <a:ext cx="3594261" cy="772794"/>
+          <a:off x="8013561" y="8461657"/>
+          <a:ext cx="3592243" cy="779566"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3354349" cy="441077"/>
         </a:xfrm>
@@ -10107,8 +10107,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7950770" y="11361615"/>
-          <a:ext cx="3610136" cy="533400"/>
+          <a:off x="7943710" y="11365938"/>
+          <a:ext cx="3608118" cy="533400"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3354349" cy="536575"/>
         </a:xfrm>
@@ -10254,8 +10254,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="8077771" y="8905525"/>
-          <a:ext cx="4410238" cy="2051509"/>
+          <a:off x="8070711" y="8887370"/>
+          <a:ext cx="4408220" cy="2083064"/>
           <a:chOff x="5203826" y="7785100"/>
           <a:chExt cx="4171950" cy="1466850"/>
         </a:xfrm>
@@ -10380,8 +10380,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13570438" y="11326690"/>
-          <a:ext cx="6387529" cy="561975"/>
+          <a:off x="13553148" y="11331013"/>
+          <a:ext cx="6405827" cy="561975"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3354349" cy="536575"/>
         </a:xfrm>
@@ -10582,8 +10582,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="18080081" y="2486311"/>
-          <a:ext cx="1932596" cy="542925"/>
+          <a:off x="18081954" y="2470461"/>
+          <a:ext cx="1931731" cy="542925"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="1808134" cy="536575"/>
         </a:xfrm>
@@ -10729,8 +10729,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="15429400" y="2487042"/>
-          <a:ext cx="2476784" cy="542925"/>
+          <a:off x="15418593" y="2471192"/>
+          <a:ext cx="2484277" cy="542925"/>
           <a:chOff x="2623745" y="1854200"/>
           <a:chExt cx="1815534" cy="536575"/>
         </a:xfrm>
@@ -11020,8 +11020,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10369329" y="989034"/>
-          <a:ext cx="2704467" cy="536575"/>
+          <a:off x="10362269" y="973328"/>
+          <a:ext cx="2702449" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
         </a:xfrm>
@@ -11475,8 +11475,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="9518620" y="1879428"/>
-          <a:ext cx="7156934" cy="3291365"/>
+          <a:off x="9511560" y="1863722"/>
+          <a:ext cx="7153187" cy="3291221"/>
           <a:chOff x="8855676" y="1884369"/>
           <a:chExt cx="6442159" cy="3287477"/>
         </a:xfrm>
@@ -13198,7 +13198,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="6061429" y="13196360"/>
+          <a:off x="6050334" y="13200683"/>
           <a:ext cx="880260" cy="240203"/>
           <a:chOff x="5992812" y="13470006"/>
           <a:chExt cx="880260" cy="370395"/>
@@ -13357,7 +13357,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4996277" y="13423777"/>
+          <a:off x="4985182" y="13428100"/>
           <a:ext cx="1944366" cy="376020"/>
           <a:chOff x="4928706" y="13473112"/>
           <a:chExt cx="1944366" cy="376020"/>
@@ -13686,7 +13686,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4996277" y="13780964"/>
+          <a:off x="4985182" y="13785287"/>
           <a:ext cx="1945953" cy="377608"/>
           <a:chOff x="4928706" y="13830299"/>
           <a:chExt cx="1945953" cy="377608"/>
@@ -14015,7 +14015,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="4996277" y="14141649"/>
+          <a:off x="4985182" y="14145972"/>
           <a:ext cx="1947033" cy="374110"/>
           <a:chOff x="4928706" y="14190984"/>
           <a:chExt cx="1947033" cy="374110"/>
@@ -14344,7 +14344,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="12226499" y="13530384"/>
+          <a:off x="12217421" y="13534707"/>
           <a:ext cx="880260" cy="240203"/>
           <a:chOff x="5992812" y="13470006"/>
           <a:chExt cx="880260" cy="370395"/>
@@ -14503,7 +14503,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="11161347" y="13757801"/>
+          <a:off x="11152269" y="13762124"/>
           <a:ext cx="1944366" cy="376020"/>
           <a:chOff x="4928706" y="13473112"/>
           <a:chExt cx="1944366" cy="376020"/>
@@ -14832,7 +14832,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="11161347" y="14114988"/>
+          <a:off x="11152269" y="14119311"/>
           <a:ext cx="1945953" cy="377608"/>
           <a:chOff x="4928706" y="13830299"/>
           <a:chExt cx="1945953" cy="377608"/>
@@ -15161,7 +15161,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="21197564" y="13164702"/>
+          <a:off x="21198572" y="13169025"/>
           <a:ext cx="880260" cy="240203"/>
           <a:chOff x="5992812" y="13470006"/>
           <a:chExt cx="880260" cy="370395"/>
@@ -15320,7 +15320,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="20132412" y="13392119"/>
+          <a:off x="20133420" y="13396442"/>
           <a:ext cx="1944366" cy="376020"/>
           <a:chOff x="4928706" y="13473112"/>
           <a:chExt cx="1944366" cy="376020"/>
@@ -15649,7 +15649,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="20132412" y="13749306"/>
+          <a:off x="20133420" y="13753629"/>
           <a:ext cx="1945953" cy="377608"/>
           <a:chOff x="4928706" y="13830299"/>
           <a:chExt cx="1945953" cy="377608"/>
@@ -15975,7 +15975,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="20132412" y="14109991"/>
+          <a:off x="20133420" y="14114314"/>
           <a:ext cx="1947033" cy="374110"/>
           <a:chOff x="4928706" y="14190984"/>
           <a:chExt cx="1947033" cy="374110"/>
@@ -16304,8 +16304,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13567531" y="3449512"/>
-          <a:ext cx="4298352" cy="4279529"/>
+          <a:off x="13550241" y="3433662"/>
+          <a:ext cx="4312328" cy="4276648"/>
           <a:chOff x="12441033" y="3461845"/>
           <a:chExt cx="3993809" cy="4282919"/>
         </a:xfrm>
@@ -17873,8 +17873,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="18275971" y="3446032"/>
-          <a:ext cx="3727686" cy="4335064"/>
+          <a:off x="18277844" y="3430182"/>
+          <a:ext cx="3726821" cy="4332183"/>
           <a:chOff x="16776161" y="3458359"/>
           <a:chExt cx="3601523" cy="4338461"/>
         </a:xfrm>
@@ -19480,7 +19480,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="932148" y="3160997"/>
+          <a:off x="921053" y="3145147"/>
           <a:ext cx="6179038" cy="2168711"/>
           <a:chOff x="932148" y="3160997"/>
           <a:chExt cx="6179038" cy="2168711"/>
@@ -19589,7 +19589,7 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>5922596</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>2692510</xdr:rowOff>
+      <xdr:rowOff>2607348</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -19604,10 +19604,10 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1164168" y="6272568"/>
-          <a:ext cx="5556249" cy="1923275"/>
+          <a:off x="1153073" y="6253837"/>
+          <a:ext cx="5556249" cy="1838113"/>
           <a:chOff x="1164168" y="6272568"/>
-          <a:chExt cx="5556249" cy="1923275"/>
+          <a:chExt cx="5556249" cy="1838113"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:pic>
@@ -19623,7 +19623,7 @@
             <a:picLocks noChangeAspect="1"/>
           </xdr:cNvPicPr>
         </xdr:nvPicPr>
-        <xdr:blipFill>
+        <xdr:blipFill rotWithShape="1">
           <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print">
             <a:extLst>
               <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
@@ -19631,14 +19631,13 @@
               </a:ext>
             </a:extLst>
           </a:blip>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
+          <a:srcRect b="4428"/>
+          <a:stretch/>
         </xdr:blipFill>
         <xdr:spPr>
           <a:xfrm>
             <a:off x="1164168" y="6272568"/>
-            <a:ext cx="5556249" cy="1923275"/>
+            <a:ext cx="5556249" cy="1838113"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>

</xml_diff>

<commit_message>
Fix: display correct numbers for estimate & throughput in metrics report
</commit_message>
<xml_diff>
--- a/assets/xlsx/visualise-metrics.xlsx
+++ b/assets/xlsx/visualise-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/workspace/sprint-metrics_webapp/assets/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03546333-04AA-184D-ACEC-22E802D93F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D4DA1E-EC48-9447-81A8-42933598C26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,9 +19,10 @@
     <sheet name="Calculated Stats" sheetId="30" r:id="rId4"/>
     <sheet name="processed | data" sheetId="29" r:id="rId5"/>
     <sheet name="rawdata | iteration analysis" sheetId="28" r:id="rId6"/>
+    <sheet name="Sheet2" sheetId="37" r:id="rId7"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <definedNames>
     <definedName name="JiraExportFileLocation">#REF!</definedName>
@@ -95,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="281">
   <si>
     <t>Done</t>
   </si>
@@ -626,6 +627,360 @@
       <t xml:space="preserve">
 (no. of items)</t>
     </r>
+  </si>
+  <si>
+    <t>labels_Convergence_count</t>
+  </si>
+  <si>
+    <t>labels_Convergence_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_Project_count</t>
+  </si>
+  <si>
+    <t>labels_Project_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_BAU_count</t>
+  </si>
+  <si>
+    <t>labels_BAU_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_FY24Q4-Committed_count</t>
+  </si>
+  <si>
+    <t>labels_FY24Q4-Committed_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_Dataverse_count</t>
+  </si>
+  <si>
+    <t>labels_Dataverse_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_HESTAi_count</t>
+  </si>
+  <si>
+    <t>labels_HESTAi_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_Improvement_count</t>
+  </si>
+  <si>
+    <t>labels_Improvement_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_Integration_count</t>
+  </si>
+  <si>
+    <t>labels_Integration_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_Cloud_count</t>
+  </si>
+  <si>
+    <t>labels_Cloud_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_DEP-Resolution_count</t>
+  </si>
+  <si>
+    <t>labels_DEP-Resolution_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_DIG-DEP.AE_count</t>
+  </si>
+  <si>
+    <t>labels_DIG-DEP.AE_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_Dep.AE_count</t>
+  </si>
+  <si>
+    <t>labels_Dep.AE_storyPoints</t>
+  </si>
+  <si>
+    <t>labels_INT-DEP.AE_count</t>
+  </si>
+  <si>
+    <t>labels_INT-DEP.AE_storyPoints</t>
+  </si>
+  <si>
+    <t>components_Dataverse_count</t>
+  </si>
+  <si>
+    <t>components_Dataverse_storyPoints</t>
+  </si>
+  <si>
+    <t>components_Architecture_count</t>
+  </si>
+  <si>
+    <t>components_Architecture_storyPoints</t>
+  </si>
+  <si>
+    <t>components_Cloud_count</t>
+  </si>
+  <si>
+    <t>components_Cloud_storyPoints</t>
+  </si>
+  <si>
+    <t>components_Partner_count</t>
+  </si>
+  <si>
+    <t>components_Partner_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_Convergence_count</t>
+  </si>
+  <si>
+    <t>completedLabels_Convergence_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_FY24Q4-Committed_count</t>
+  </si>
+  <si>
+    <t>completedLabels_FY24Q4-Committed_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_BAU_count</t>
+  </si>
+  <si>
+    <t>completedLabels_BAU_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_Dataverse_count</t>
+  </si>
+  <si>
+    <t>completedLabels_Dataverse_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_Project_count</t>
+  </si>
+  <si>
+    <t>completedLabels_Project_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_Improvement_count</t>
+  </si>
+  <si>
+    <t>completedLabels_Improvement_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_DEP-Resolution_count</t>
+  </si>
+  <si>
+    <t>completedLabels_DEP-Resolution_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_DIG-DEP.AE_count</t>
+  </si>
+  <si>
+    <t>completedLabels_DIG-DEP.AE_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_Dep.AE_count</t>
+  </si>
+  <si>
+    <t>completedLabels_Dep.AE_storyPoints</t>
+  </si>
+  <si>
+    <t>completedLabels_INT-DEP.AE_count</t>
+  </si>
+  <si>
+    <t>completedLabels_INT-DEP.AE_storyPoints</t>
+  </si>
+  <si>
+    <t>completedComponents_Dataverse_count</t>
+  </si>
+  <si>
+    <t>completedComponents_Dataverse_storyPoints</t>
+  </si>
+  <si>
+    <t>completedComponents_Cloud_count</t>
+  </si>
+  <si>
+    <t>completedComponents_Cloud_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Cloud Infra &amp; DevOps (BAU)_count</t>
+  </si>
+  <si>
+    <t>parents_Cloud Infra &amp; DevOps (BAU)_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Visualisation Layer from Dataverse_count</t>
+  </si>
+  <si>
+    <t>parents_Visualisation Layer from Dataverse_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Dataverse Readiness for Convergence_count</t>
+  </si>
+  <si>
+    <t>parents_Dataverse Readiness for Convergence_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Improvement | AWS Platform (FY24Q4)_count</t>
+  </si>
+  <si>
+    <t>parents_Improvement | AWS Platform (FY24Q4)_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Data governance support_count</t>
+  </si>
+  <si>
+    <t>parents_Data governance support_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_GROW Data Ingestion - Incremental load_count</t>
+  </si>
+  <si>
+    <t>parents_GROW Data Ingestion - Incremental load_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_IDS - DAA Cockpit | Cloud_count</t>
+  </si>
+  <si>
+    <t>parents_IDS - DAA Cockpit | Cloud_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Event Based Stream for non-prod_count</t>
+  </si>
+  <si>
+    <t>parents_Event Based Stream for non-prod_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Identity Federation | PoC_count</t>
+  </si>
+  <si>
+    <t>parents_Identity Federation | PoC_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Identity Federation | Go Live_count</t>
+  </si>
+  <si>
+    <t>parents_Identity Federation | Go Live_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Investments Architecture Support_count</t>
+  </si>
+  <si>
+    <t>parents_Investments Architecture Support_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Cloud Infrastructure for all channels (PROD)_count</t>
+  </si>
+  <si>
+    <t>parents_Cloud Infrastructure for all channels (PROD)_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Modern Management Architecture_count</t>
+  </si>
+  <si>
+    <t>parents_Modern Management Architecture_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Convergence_count</t>
+  </si>
+  <si>
+    <t>parents_Convergence_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_BAU | Architecture Security - ARFS &amp; Reviews_count</t>
+  </si>
+  <si>
+    <t>parents_BAU | Architecture Security - ARFS &amp; Reviews_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_HESTAi - Redactive AI PoC_count</t>
+  </si>
+  <si>
+    <t>parents_HESTAi - Redactive AI PoC_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_HESTAi - Statements QA Automation_count</t>
+  </si>
+  <si>
+    <t>parents_HESTAi - Statements QA Automation_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Digital Architecture Q4_count</t>
+  </si>
+  <si>
+    <t>parents_Digital Architecture Q4_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_BAU | Cloud Infra &amp; DevOps (FY24Q4)_count</t>
+  </si>
+  <si>
+    <t>parents_BAU | Cloud Infra &amp; DevOps (FY24Q4)_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_BAU | Cloud Data Support (FY24Q4)_count</t>
+  </si>
+  <si>
+    <t>parents_BAU | Cloud Data Support (FY24Q4)_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Improvement | Dataverse Enhancements (FY24Q4)_count</t>
+  </si>
+  <si>
+    <t>parents_Improvement | Dataverse Enhancements (FY24Q4)_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_IDS - DAA Cockpit | Dataverse_count</t>
+  </si>
+  <si>
+    <t>parents_IDS - DAA Cockpit | Dataverse_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Data Servicing for IDS_count</t>
+  </si>
+  <si>
+    <t>parents_Data Servicing for IDS_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Replacement for Digital SMS providor_count</t>
+  </si>
+  <si>
+    <t>parents_Replacement for Digital SMS providor_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_Future planner changes July 1 2024_count</t>
+  </si>
+  <si>
+    <t>parents_Future planner changes July 1 2024_storyPoints</t>
+  </si>
+  <si>
+    <t>parents_undefined_count</t>
+  </si>
+  <si>
+    <t>parents_undefined_storyPoints</t>
+  </si>
+  <si>
+    <t>emergentWork_count</t>
+  </si>
+  <si>
+    <t>emergentWork_storyPoints</t>
+  </si>
+  <si>
+    <t>sprintPlanning_targetCapacity_throughput</t>
+  </si>
+  <si>
+    <t>trends_velocityTrends_throughput</t>
+  </si>
+  <si>
+    <t>insights_achievableSprintGoal_throughput</t>
+  </si>
+  <si>
+    <t>insights_healthyPerformanceTarget_throughput</t>
+  </si>
+  <si>
+    <t>#1</t>
+  </si>
+  <si>
+    <t>ACME Squad</t>
   </si>
 </sst>
 </file>
@@ -18325,7 +18680,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="863614" y="2487503"/>
+          <a:off x="855147" y="2466336"/>
           <a:ext cx="2438064" cy="601889"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
@@ -18489,7 +18844,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="895227" y="6223457"/>
+          <a:off x="886760" y="6189590"/>
           <a:ext cx="2692153" cy="575912"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2679967" cy="536575"/>
@@ -18866,8 +19221,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="871500" y="3232497"/>
-          <a:ext cx="6098382" cy="2571544"/>
+          <a:off x="863033" y="3211330"/>
+          <a:ext cx="6094149" cy="2563078"/>
           <a:chOff x="932148" y="3160997"/>
           <a:chExt cx="6179038" cy="2168711"/>
         </a:xfrm>
@@ -18990,8 +19345,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1358462" y="7352576"/>
-          <a:ext cx="5688244" cy="2080680"/>
+          <a:off x="1349995" y="7314476"/>
+          <a:ext cx="5688244" cy="2025647"/>
           <a:chOff x="1164168" y="6272568"/>
           <a:chExt cx="5556249" cy="1838113"/>
         </a:xfrm>
@@ -19244,8 +19599,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="16828437" y="2510742"/>
-          <a:ext cx="1947483" cy="531433"/>
+          <a:off x="16794570" y="2489575"/>
+          <a:ext cx="1934783" cy="531433"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="1808134" cy="536575"/>
         </a:xfrm>
@@ -19391,8 +19746,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13742814" y="2511473"/>
-          <a:ext cx="2931265" cy="531433"/>
+          <a:off x="13721647" y="2490306"/>
+          <a:ext cx="2918565" cy="531433"/>
           <a:chOff x="2623745" y="1854200"/>
           <a:chExt cx="1815534" cy="536575"/>
         </a:xfrm>
@@ -19540,8 +19895,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="12414632" y="3238931"/>
-          <a:ext cx="4327033" cy="3861018"/>
+          <a:off x="12397699" y="3217764"/>
+          <a:ext cx="4310099" cy="3848318"/>
           <a:chOff x="12441033" y="3461845"/>
           <a:chExt cx="3993809" cy="4282919"/>
         </a:xfrm>
@@ -19769,7 +20124,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!R23">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!R22">
           <xdr:nvSpPr>
             <xdr:cNvPr id="36" name="TextBox 35">
               <a:extLst>
@@ -19814,7 +20169,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{2F14E553-9C0A-42F7-ADE5-4DBB4C5CE298}" type="TxLink">
+              <a:fld id="{D20803C0-A93E-0E4F-AE2B-AC5D5DF6171C}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -19837,7 +20192,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!#REF!">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!R23">
           <xdr:nvSpPr>
             <xdr:cNvPr id="37" name="TextBox 36">
               <a:extLst>
@@ -19882,7 +20237,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{B7CEC906-7727-4607-8207-F44889F61CAA}" type="TxLink">
+              <a:fld id="{D927C692-535C-6746-845B-21D87C83B062}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -21109,8 +21464,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="16946474" y="3224039"/>
-          <a:ext cx="3739283" cy="3945010"/>
+          <a:off x="16912607" y="3202872"/>
+          <a:ext cx="3726583" cy="3932310"/>
           <a:chOff x="16776161" y="3461534"/>
           <a:chExt cx="3598348" cy="4370066"/>
         </a:xfrm>
@@ -21283,7 +21638,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="14015005" y="5918697"/>
+              <a:off x="14015005" y="5909304"/>
               <a:ext cx="1211676" cy="588956"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -21338,7 +21693,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!T23">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!T22">
           <xdr:nvSpPr>
             <xdr:cNvPr id="64" name="TextBox 63">
               <a:extLst>
@@ -21351,8 +21706,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="15245705" y="5933266"/>
-              <a:ext cx="1198273" cy="588956"/>
+              <a:off x="15245705" y="5923873"/>
+              <a:ext cx="1198273" cy="588702"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -21383,7 +21738,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{9A7E5D21-B262-4C68-A205-5ED5ED046BA7}" type="TxLink">
+              <a:fld id="{329C7112-1040-D14A-BA44-E45B2BB4AFDD}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -21406,7 +21761,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!#REF!">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!T23">
           <xdr:nvSpPr>
             <xdr:cNvPr id="65" name="TextBox 64">
               <a:extLst>
@@ -21419,8 +21774,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="16440288" y="5936716"/>
-              <a:ext cx="1156607" cy="588956"/>
+              <a:off x="16440288" y="5917930"/>
+              <a:ext cx="1156607" cy="588702"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -21451,7 +21806,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{7D0047C9-7AA8-4997-A893-F0251AA2C29B}" type="TxLink">
+              <a:fld id="{6758FAC0-9153-8846-9EB5-694813C3E9F9}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -22266,8 +22621,8 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="5400000" flipH="1" flipV="1">
-              <a:off x="14813791" y="4890959"/>
-              <a:ext cx="834789" cy="1220686"/>
+              <a:off x="14818488" y="4886264"/>
+              <a:ext cx="825396" cy="1220686"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
               <a:avLst>
@@ -22309,8 +22664,8 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="16200000" flipV="1">
-              <a:off x="15418507" y="5506930"/>
-              <a:ext cx="849359" cy="3312"/>
+              <a:off x="15423203" y="5502234"/>
+              <a:ext cx="839966" cy="3312"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
               <a:avLst>
@@ -22352,8 +22707,8 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="16200000" flipH="1">
-              <a:off x="16003657" y="4921779"/>
-              <a:ext cx="852809" cy="1177063"/>
+              <a:off x="16013049" y="4912387"/>
+              <a:ext cx="834023" cy="1177062"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
               <a:avLst>
@@ -22678,8 +23033,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="9873279" y="2536177"/>
-          <a:ext cx="2699867" cy="536575"/>
+          <a:off x="9856346" y="2515010"/>
+          <a:ext cx="2691400" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
         </a:xfrm>
@@ -22825,7 +23180,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7137182" y="2525853"/>
+          <a:off x="7128715" y="2504686"/>
           <a:ext cx="2403472" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2394604" cy="536575"/>
@@ -23465,8 +23820,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7203803" y="6456564"/>
-          <a:ext cx="4944657" cy="3418208"/>
+          <a:off x="7195336" y="6422697"/>
+          <a:ext cx="4936191" cy="3342008"/>
           <a:chOff x="900706" y="5293038"/>
           <a:chExt cx="4942746" cy="3405917"/>
         </a:xfrm>
@@ -23620,7 +23975,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="7177494" y="6222782"/>
+          <a:off x="7169027" y="6188915"/>
           <a:ext cx="2466973" cy="536575"/>
           <a:chOff x="1920877" y="1854200"/>
           <a:chExt cx="2470148" cy="536575"/>
@@ -23788,8 +24143,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="890971" y="9772274"/>
-          <a:ext cx="3325427" cy="765210"/>
+          <a:off x="882504" y="9662207"/>
+          <a:ext cx="3321194" cy="765210"/>
           <a:chOff x="1920876" y="1854200"/>
           <a:chExt cx="3319649" cy="433685"/>
         </a:xfrm>
@@ -24026,8 +24381,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="9118769" y="3972933"/>
-          <a:ext cx="6340373" cy="3077811"/>
+          <a:off x="9110302" y="3951766"/>
+          <a:ext cx="6319207" cy="3065111"/>
           <a:chOff x="9118769" y="3955999"/>
           <a:chExt cx="6323440" cy="3069345"/>
         </a:xfrm>
@@ -24290,8 +24645,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="10138165" y="3867576"/>
-          <a:ext cx="2471180" cy="1180482"/>
+          <a:off x="10121232" y="3846409"/>
+          <a:ext cx="2462713" cy="1172016"/>
           <a:chOff x="10122851" y="3844436"/>
           <a:chExt cx="2462005" cy="1169688"/>
         </a:xfrm>
@@ -26404,7 +26759,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!R23">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!R22">
           <xdr:nvSpPr>
             <xdr:cNvPr id="36" name="TextBox 35">
               <a:extLst>
@@ -26449,7 +26804,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{2F14E553-9C0A-42F7-ADE5-4DBB4C5CE298}" type="TxLink">
+              <a:fld id="{7D59C68A-89B0-F748-B43E-601993CB5D28}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -26472,7 +26827,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!#REF!">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!R23">
           <xdr:nvSpPr>
             <xdr:cNvPr id="37" name="TextBox 36">
               <a:extLst>
@@ -26517,7 +26872,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{B7CEC906-7727-4607-8207-F44889F61CAA}" type="TxLink">
+              <a:fld id="{2C6ACE09-2A82-F84E-B40C-6E0844DA0055}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -27973,7 +28328,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!T23">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!T22">
           <xdr:nvSpPr>
             <xdr:cNvPr id="64" name="TextBox 63">
               <a:extLst>
@@ -27987,7 +28342,7 @@
           <xdr:spPr>
             <a:xfrm>
               <a:off x="15245705" y="5933266"/>
-              <a:ext cx="1198273" cy="588956"/>
+              <a:ext cx="1198273" cy="589336"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -28018,7 +28373,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{9A7E5D21-B262-4C68-A205-5ED5ED046BA7}" type="TxLink">
+              <a:fld id="{D12BBEA6-9179-7943-B327-AEB365E0EA5C}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -28041,7 +28396,7 @@
             </a:p>
           </xdr:txBody>
         </xdr:sp>
-        <xdr:sp macro="" textlink="'Sprint Summary | data'!#REF!">
+        <xdr:sp macro="" textlink="'Sprint Summary | data'!T23">
           <xdr:nvSpPr>
             <xdr:cNvPr id="65" name="TextBox 64">
               <a:extLst>
@@ -28054,8 +28409,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="16440288" y="5936716"/>
-              <a:ext cx="1156607" cy="588956"/>
+              <a:off x="16440288" y="5936717"/>
+              <a:ext cx="1156607" cy="589336"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -28086,7 +28441,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr marL="0" indent="0" algn="ctr"/>
-              <a:fld id="{7D0047C9-7AA8-4997-A893-F0251AA2C29B}" type="TxLink">
+              <a:fld id="{DA8D4262-FA89-AC41-B211-D75B251186AC}" type="TxLink">
                 <a:rPr lang="en-US" sz="2800" b="0" i="0" u="none" strike="noStrike">
                   <a:solidFill>
                     <a:srgbClr val="000000"/>
@@ -28944,7 +29299,7 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="16200000" flipV="1">
-              <a:off x="15418507" y="5506930"/>
+              <a:off x="15418507" y="5506931"/>
               <a:ext cx="849359" cy="3312"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
@@ -28987,7 +29342,7 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="16200000" flipH="1">
-              <a:off x="16003657" y="4921779"/>
+              <a:off x="16003656" y="4921781"/>
               <a:ext cx="852809" cy="1177063"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
@@ -47897,10 +48252,10 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:EN2"/>
+  <dimension ref="A1:EZ2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:144" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:156" x14ac:dyDescent="0.2">
       <c r="A1" s="90"/>
       <c r="B1" s="90"/>
       <c r="C1" s="90"/>
@@ -48045,8 +48400,20 @@
       <c r="EL1" s="90"/>
       <c r="EM1" s="90"/>
       <c r="EN1" s="90"/>
-    </row>
-    <row r="2" spans="1:144" x14ac:dyDescent="0.2">
+      <c r="EO1" s="90"/>
+      <c r="EP1" s="90"/>
+      <c r="EQ1" s="90"/>
+      <c r="ER1" s="90"/>
+      <c r="ES1" s="90"/>
+      <c r="ET1" s="90"/>
+      <c r="EU1" s="90"/>
+      <c r="EV1" s="90"/>
+      <c r="EW1" s="90"/>
+      <c r="EX1" s="90"/>
+      <c r="EY1" s="90"/>
+      <c r="EZ1" s="90"/>
+    </row>
+    <row r="2" spans="1:156" x14ac:dyDescent="0.2">
       <c r="A2" s="90"/>
       <c r="B2" s="91"/>
       <c r="C2" s="96"/>
@@ -48191,6 +48558,1183 @@
       <c r="EL2" s="91"/>
       <c r="EM2" s="91"/>
       <c r="EN2" s="91"/>
+      <c r="EO2" s="91"/>
+      <c r="EP2" s="91"/>
+      <c r="EQ2" s="91"/>
+      <c r="ER2" s="91"/>
+      <c r="ES2" s="91"/>
+      <c r="ET2" s="91"/>
+      <c r="EU2" s="91"/>
+      <c r="EV2" s="91"/>
+      <c r="EW2" s="91"/>
+      <c r="EX2" s="91"/>
+      <c r="EY2" s="91"/>
+      <c r="EZ2" s="91"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{752FB2B1-D370-8640-913E-87A21EE3986A}">
+  <dimension ref="A1:B144"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="96.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="90" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="90" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="90" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="91" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="90" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" s="96">
+        <v>36892</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="90" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="96">
+        <v>37289</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="90" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="91">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="90" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="91">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="90" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="91">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="90" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="91">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="90" t="s">
+        <v>96</v>
+      </c>
+      <c r="B9" s="91">
+        <v>69.75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="90" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="91">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="90" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="91">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="90" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="91">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="90" t="s">
+        <v>100</v>
+      </c>
+      <c r="B13" s="91">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="90" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="91">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="90" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" s="91">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="90" t="s">
+        <v>103</v>
+      </c>
+      <c r="B16" s="91">
+        <v>33.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="90" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" s="91">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="90" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" s="91">
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="90" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="91">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="90" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" s="91">
+        <v>15.25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="90" t="s">
+        <v>163</v>
+      </c>
+      <c r="B21" s="91">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="90" t="s">
+        <v>164</v>
+      </c>
+      <c r="B22" s="91">
+        <v>23.25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="90" t="s">
+        <v>165</v>
+      </c>
+      <c r="B23" s="91">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="90" t="s">
+        <v>166</v>
+      </c>
+      <c r="B24" s="91">
+        <v>35.75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="90" t="s">
+        <v>167</v>
+      </c>
+      <c r="B25" s="91">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="90" t="s">
+        <v>168</v>
+      </c>
+      <c r="B26" s="91">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="90" t="s">
+        <v>169</v>
+      </c>
+      <c r="B27" s="91">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="90" t="s">
+        <v>170</v>
+      </c>
+      <c r="B28" s="91">
+        <v>47.25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="90" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="90" t="s">
+        <v>172</v>
+      </c>
+      <c r="B30" s="91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="90" t="s">
+        <v>173</v>
+      </c>
+      <c r="B31" s="91">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="90" t="s">
+        <v>174</v>
+      </c>
+      <c r="B32" s="91">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="90" t="s">
+        <v>175</v>
+      </c>
+      <c r="B33" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="90" t="s">
+        <v>176</v>
+      </c>
+      <c r="B34" s="91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="90" t="s">
+        <v>177</v>
+      </c>
+      <c r="B35" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="90" t="s">
+        <v>178</v>
+      </c>
+      <c r="B36" s="91">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="90" t="s">
+        <v>179</v>
+      </c>
+      <c r="B37" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="90" t="s">
+        <v>180</v>
+      </c>
+      <c r="B38" s="91">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="90" t="s">
+        <v>181</v>
+      </c>
+      <c r="B39" s="91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="90" t="s">
+        <v>182</v>
+      </c>
+      <c r="B40" s="91">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="90" t="s">
+        <v>183</v>
+      </c>
+      <c r="B41" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="90" t="s">
+        <v>184</v>
+      </c>
+      <c r="B42" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="90" t="s">
+        <v>185</v>
+      </c>
+      <c r="B43" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="90" t="s">
+        <v>186</v>
+      </c>
+      <c r="B44" s="91">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="90" t="s">
+        <v>187</v>
+      </c>
+      <c r="B45" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="90" t="s">
+        <v>188</v>
+      </c>
+      <c r="B46" s="91">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="90" t="s">
+        <v>189</v>
+      </c>
+      <c r="B47" s="91">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="90" t="s">
+        <v>190</v>
+      </c>
+      <c r="B48" s="91">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="90" t="s">
+        <v>191</v>
+      </c>
+      <c r="B49" s="91">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="90" t="s">
+        <v>192</v>
+      </c>
+      <c r="B50" s="91">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="90" t="s">
+        <v>193</v>
+      </c>
+      <c r="B51" s="91">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="90" t="s">
+        <v>194</v>
+      </c>
+      <c r="B52" s="91">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="90" t="s">
+        <v>195</v>
+      </c>
+      <c r="B53" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="90" t="s">
+        <v>196</v>
+      </c>
+      <c r="B54" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="90" t="s">
+        <v>197</v>
+      </c>
+      <c r="B55" s="91">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="90" t="s">
+        <v>198</v>
+      </c>
+      <c r="B56" s="91">
+        <v>7.25</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="90" t="s">
+        <v>199</v>
+      </c>
+      <c r="B57" s="91">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="90" t="s">
+        <v>200</v>
+      </c>
+      <c r="B58" s="91">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="90" t="s">
+        <v>201</v>
+      </c>
+      <c r="B59" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="90" t="s">
+        <v>202</v>
+      </c>
+      <c r="B60" s="91">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="90" t="s">
+        <v>203</v>
+      </c>
+      <c r="B61" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="90" t="s">
+        <v>204</v>
+      </c>
+      <c r="B62" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="90" t="s">
+        <v>205</v>
+      </c>
+      <c r="B63" s="91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" s="90" t="s">
+        <v>206</v>
+      </c>
+      <c r="B64" s="91">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" s="90" t="s">
+        <v>207</v>
+      </c>
+      <c r="B65" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" s="90" t="s">
+        <v>208</v>
+      </c>
+      <c r="B66" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="90" t="s">
+        <v>209</v>
+      </c>
+      <c r="B67" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="90" t="s">
+        <v>210</v>
+      </c>
+      <c r="B68" s="91">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="90" t="s">
+        <v>211</v>
+      </c>
+      <c r="B69" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="90" t="s">
+        <v>212</v>
+      </c>
+      <c r="B70" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="90" t="s">
+        <v>213</v>
+      </c>
+      <c r="B71" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" s="90" t="s">
+        <v>214</v>
+      </c>
+      <c r="B72" s="91">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="90" t="s">
+        <v>215</v>
+      </c>
+      <c r="B73" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="90" t="s">
+        <v>216</v>
+      </c>
+      <c r="B74" s="91">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="90" t="s">
+        <v>217</v>
+      </c>
+      <c r="B75" s="91">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="90" t="s">
+        <v>218</v>
+      </c>
+      <c r="B76" s="91">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="90" t="s">
+        <v>219</v>
+      </c>
+      <c r="B77" s="91">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="90" t="s">
+        <v>220</v>
+      </c>
+      <c r="B78" s="91">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" s="90" t="s">
+        <v>221</v>
+      </c>
+      <c r="B79" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="90" t="s">
+        <v>222</v>
+      </c>
+      <c r="B80" s="91">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" s="90" t="s">
+        <v>223</v>
+      </c>
+      <c r="B81" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" s="90" t="s">
+        <v>224</v>
+      </c>
+      <c r="B82" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" s="90" t="s">
+        <v>225</v>
+      </c>
+      <c r="B83" s="91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" s="90" t="s">
+        <v>226</v>
+      </c>
+      <c r="B84" s="91">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" s="90" t="s">
+        <v>227</v>
+      </c>
+      <c r="B85" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" s="90" t="s">
+        <v>228</v>
+      </c>
+      <c r="B86" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" s="90" t="s">
+        <v>229</v>
+      </c>
+      <c r="B87" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" s="90" t="s">
+        <v>230</v>
+      </c>
+      <c r="B88" s="91">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" s="90" t="s">
+        <v>231</v>
+      </c>
+      <c r="B89" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" s="90" t="s">
+        <v>232</v>
+      </c>
+      <c r="B90" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" s="90" t="s">
+        <v>233</v>
+      </c>
+      <c r="B91" s="91">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92" s="90" t="s">
+        <v>234</v>
+      </c>
+      <c r="B92" s="91">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A93" s="90" t="s">
+        <v>235</v>
+      </c>
+      <c r="B93" s="91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A94" s="90" t="s">
+        <v>236</v>
+      </c>
+      <c r="B94" s="91">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A95" s="90" t="s">
+        <v>237</v>
+      </c>
+      <c r="B95" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A96" s="90" t="s">
+        <v>238</v>
+      </c>
+      <c r="B96" s="91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" s="90" t="s">
+        <v>239</v>
+      </c>
+      <c r="B97" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" s="90" t="s">
+        <v>240</v>
+      </c>
+      <c r="B98" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" s="90" t="s">
+        <v>241</v>
+      </c>
+      <c r="B99" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" s="90" t="s">
+        <v>242</v>
+      </c>
+      <c r="B100" s="91">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" s="90" t="s">
+        <v>243</v>
+      </c>
+      <c r="B101" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102" s="90" t="s">
+        <v>244</v>
+      </c>
+      <c r="B102" s="91">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103" s="90" t="s">
+        <v>245</v>
+      </c>
+      <c r="B103" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A104" s="90" t="s">
+        <v>246</v>
+      </c>
+      <c r="B104" s="91">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A105" s="90" t="s">
+        <v>247</v>
+      </c>
+      <c r="B105" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A106" s="90" t="s">
+        <v>248</v>
+      </c>
+      <c r="B106" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A107" s="90" t="s">
+        <v>249</v>
+      </c>
+      <c r="B107" s="91">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A108" s="90" t="s">
+        <v>250</v>
+      </c>
+      <c r="B108" s="91">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A109" s="90" t="s">
+        <v>251</v>
+      </c>
+      <c r="B109" s="91">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A110" s="90" t="s">
+        <v>252</v>
+      </c>
+      <c r="B110" s="91">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111" s="90" t="s">
+        <v>253</v>
+      </c>
+      <c r="B111" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" s="90" t="s">
+        <v>254</v>
+      </c>
+      <c r="B112" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113" s="90" t="s">
+        <v>255</v>
+      </c>
+      <c r="B113" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114" s="90" t="s">
+        <v>256</v>
+      </c>
+      <c r="B114" s="91">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A115" s="90" t="s">
+        <v>257</v>
+      </c>
+      <c r="B115" s="91">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A116" s="90" t="s">
+        <v>258</v>
+      </c>
+      <c r="B116" s="91">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A117" s="90" t="s">
+        <v>259</v>
+      </c>
+      <c r="B117" s="91">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A118" s="90" t="s">
+        <v>260</v>
+      </c>
+      <c r="B118" s="91">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A119" s="90" t="s">
+        <v>261</v>
+      </c>
+      <c r="B119" s="91">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A120" s="90" t="s">
+        <v>262</v>
+      </c>
+      <c r="B120" s="91">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A121" s="90" t="s">
+        <v>263</v>
+      </c>
+      <c r="B121" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A122" s="90" t="s">
+        <v>264</v>
+      </c>
+      <c r="B122" s="91">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A123" s="90" t="s">
+        <v>265</v>
+      </c>
+      <c r="B123" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A124" s="90" t="s">
+        <v>266</v>
+      </c>
+      <c r="B124" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A125" s="90" t="s">
+        <v>267</v>
+      </c>
+      <c r="B125" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A126" s="90" t="s">
+        <v>268</v>
+      </c>
+      <c r="B126" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A127" s="90" t="s">
+        <v>269</v>
+      </c>
+      <c r="B127" s="91">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A128" s="90" t="s">
+        <v>270</v>
+      </c>
+      <c r="B128" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A129" s="90" t="s">
+        <v>271</v>
+      </c>
+      <c r="B129" s="91">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A130" s="90" t="s">
+        <v>272</v>
+      </c>
+      <c r="B130" s="91">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A131" s="90" t="s">
+        <v>273</v>
+      </c>
+      <c r="B131" s="91">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A132" s="90" t="s">
+        <v>274</v>
+      </c>
+      <c r="B132" s="91">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A133" s="90" t="s">
+        <v>108</v>
+      </c>
+      <c r="B133" s="91">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A134" s="90" t="s">
+        <v>150</v>
+      </c>
+      <c r="B134" s="91">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A135" s="90" t="s">
+        <v>109</v>
+      </c>
+      <c r="B135" s="91">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A136" s="90" t="s">
+        <v>110</v>
+      </c>
+      <c r="B136" s="91">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A137" s="90" t="s">
+        <v>111</v>
+      </c>
+      <c r="B137" s="91">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A138" s="90" t="s">
+        <v>275</v>
+      </c>
+      <c r="B138" s="91">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A139" s="90" t="s">
+        <v>112</v>
+      </c>
+      <c r="B139" s="91">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A140" s="90" t="s">
+        <v>276</v>
+      </c>
+      <c r="B140" s="91">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A141" s="90" t="s">
+        <v>113</v>
+      </c>
+      <c r="B141" s="91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A142" s="90" t="s">
+        <v>277</v>
+      </c>
+      <c r="B142" s="91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A143" s="90" t="s">
+        <v>114</v>
+      </c>
+      <c r="B143" s="91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A144" s="90" t="s">
+        <v>278</v>
+      </c>
+      <c r="B144" s="91" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fix: Symbol in table for estimate/throughput should (+) for committed at start of sprint
</commit_message>
<xml_diff>
--- a/assets/xlsx/visualise-metrics.xlsx
+++ b/assets/xlsx/visualise-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/workspace/sprint-metrics_webapp/assets/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D4DA1E-EC48-9447-81A8-42933598C26F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D58F707-7C17-8D43-BDAF-1D9A348601BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -273,9 +273,6 @@
   </si>
   <si>
     <t>removed from sprint (-)</t>
-  </si>
-  <si>
-    <t>committed at sprint start (-)</t>
   </si>
   <si>
     <t>incomplete</t>
@@ -981,6 +978,9 @@
   </si>
   <si>
     <t>ACME Squad</t>
+  </si>
+  <si>
+    <t>committed at sprint start (+)</t>
   </si>
 </sst>
 </file>
@@ -36765,11 +36765,11 @@
       <c r="G8" s="104"/>
       <c r="H8" s="105"/>
       <c r="I8" s="133" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J8" s="133"/>
       <c r="K8" s="133" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L8" s="133"/>
       <c r="M8" s="106"/>
@@ -36876,7 +36876,7 @@
       <c r="F12" s="132"/>
       <c r="G12" s="104"/>
       <c r="H12" s="113" t="s">
-        <v>59</v>
+        <v>280</v>
       </c>
       <c r="I12" s="116">
         <f>'Sprint Summary | data'!R21</f>
@@ -37202,11 +37202,11 @@
       <c r="G8" s="104"/>
       <c r="H8" s="105"/>
       <c r="I8" s="133" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J8" s="133"/>
       <c r="K8" s="133" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L8" s="133"/>
       <c r="M8" s="106"/>
@@ -37313,7 +37313,7 @@
       <c r="F12" s="132"/>
       <c r="G12" s="104"/>
       <c r="H12" s="113" t="s">
-        <v>59</v>
+        <v>280</v>
       </c>
       <c r="I12" s="116">
         <f>'Sprint Summary | data'!R21</f>
@@ -37535,12 +37535,12 @@
   <sheetData>
     <row r="1" spans="1:24" s="41" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A1" s="41" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:24" s="37" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.2">
@@ -37564,7 +37564,7 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B5" s="4">
         <f>'Calculated Stats'!C22</f>
@@ -37623,7 +37623,7 @@
       <c r="G8" s="4"/>
       <c r="H8"/>
       <c r="M8" s="26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N8" s="25"/>
       <c r="O8" s="25"/>
@@ -37640,7 +37640,7 @@
       <c r="G9" s="4"/>
       <c r="H9"/>
       <c r="M9" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="N9" s="4">
         <f>'Calculated Stats'!C143</f>
@@ -37899,7 +37899,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="I20" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J20" s="4">
         <f>'Calculated Stats'!C106</f>
@@ -38091,7 +38091,7 @@
       <c r="N26" s="4"/>
       <c r="O26" s="4"/>
       <c r="Q26" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="R26" s="26"/>
       <c r="S26" s="26"/>
@@ -38102,7 +38102,7 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B27" s="4">
         <f>SUM(B29:B31)</f>
@@ -38131,7 +38131,7 @@
     <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" s="4"/>
       <c r="B28" s="34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C28" s="34" t="s">
         <v>7</v>
@@ -38148,7 +38148,7 @@
       <c r="N28" s="4"/>
       <c r="O28" s="4"/>
       <c r="Q28" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="R28" s="4">
         <f>'Calculated Stats'!C146</f>
@@ -38187,7 +38187,7 @@
       <c r="N29" s="4"/>
       <c r="O29" s="4"/>
       <c r="Q29" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="R29" s="4">
         <f>'Calculated Stats'!C145</f>
@@ -38334,7 +38334,7 @@
       <c r="N38" s="4"/>
       <c r="O38" s="4"/>
       <c r="Q38" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="R38" s="4">
         <f>SUM(R40:R44)</f>
@@ -38450,7 +38450,7 @@
     </row>
     <row r="43" spans="9:23" x14ac:dyDescent="0.2">
       <c r="I43" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J43" s="4">
         <f>'Calculated Stats'!E107</f>
@@ -38471,7 +38471,7 @@
     </row>
     <row r="44" spans="9:23" x14ac:dyDescent="0.2">
       <c r="I44" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J44" s="4">
         <f>'Calculated Stats'!C107</f>
@@ -38553,7 +38553,7 @@
     </row>
     <row r="52" spans="9:15" x14ac:dyDescent="0.2">
       <c r="I52" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J52" s="4">
         <f>'Calculated Stats'!C136</f>
@@ -38567,7 +38567,7 @@
     </row>
     <row r="53" spans="9:15" x14ac:dyDescent="0.2">
       <c r="I53" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J53" s="4">
         <f>'Calculated Stats'!E108</f>
@@ -38627,7 +38627,7 @@
     </row>
     <row r="60" spans="9:15" x14ac:dyDescent="0.2">
       <c r="I60" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J60" s="4">
         <f>'Calculated Stats'!C124</f>
@@ -38653,7 +38653,7 @@
     </row>
     <row r="62" spans="9:15" x14ac:dyDescent="0.2">
       <c r="I62" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="J62" s="4">
         <f>'Calculated Stats'!E107</f>
@@ -38667,7 +38667,7 @@
     </row>
     <row r="63" spans="9:15" x14ac:dyDescent="0.2">
       <c r="I63" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J63" s="4">
         <f>'Calculated Stats'!C107</f>
@@ -38737,7 +38737,7 @@
     </row>
     <row r="72" spans="9:15" x14ac:dyDescent="0.2">
       <c r="I72" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J72" s="4">
         <f>'Calculated Stats'!C130</f>
@@ -38852,12 +38852,12 @@
   <sheetData>
     <row r="1" spans="2:7" s="39" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="B1" s="40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="2:7" s="42" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B2" s="42" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F2" s="43"/>
     </row>
@@ -38887,7 +38887,7 @@
     </row>
     <row r="6" spans="2:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="134" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C6" s="135"/>
       <c r="D6" s="85"/>
@@ -38897,10 +38897,10 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B7" s="55" t="s">
+        <v>114</v>
+      </c>
+      <c r="C7" s="58" t="s">
         <v>115</v>
-      </c>
-      <c r="C7" s="58" t="s">
-        <v>116</v>
       </c>
       <c r="D7" s="85"/>
       <c r="E7" s="85"/>
@@ -38912,7 +38912,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="59" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D8" s="85"/>
       <c r="E8" s="85"/>
@@ -38924,7 +38924,7 @@
         <v>53</v>
       </c>
       <c r="C9" s="59" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D9" s="85"/>
       <c r="E9" s="85"/>
@@ -38933,10 +38933,10 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="56" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C10" s="59" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D10" s="85"/>
       <c r="E10" s="85"/>
@@ -38945,7 +38945,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="56" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C11" s="59"/>
       <c r="D11" s="85"/>
@@ -39043,7 +39043,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="77" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C20" s="77"/>
       <c r="D20" s="85"/>
@@ -39053,7 +39053,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C21" s="11">
         <f>'processed | data'!B6</f>
@@ -39066,7 +39066,7 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C22" s="11">
         <f>'processed | data'!B7</f>
@@ -39079,7 +39079,7 @@
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C23" s="11" t="str">
         <f>TEXT('processed | data'!B8, "DD/MM/YYYY")</f>
@@ -39092,7 +39092,7 @@
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C24" s="11" t="str">
         <f>TEXT('processed | data'!B9, "DD/MM/YYYY")</f>
@@ -39161,7 +39161,7 @@
     </row>
     <row r="32" spans="2:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="134" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C32" s="135"/>
       <c r="D32" s="28"/>
@@ -39193,7 +39193,7 @@
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B35" s="61" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C35" s="52" t="s">
         <v>40</v>
@@ -39418,7 +39418,7 @@
         <v>26</v>
       </c>
       <c r="C49" s="139" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D49" s="139"/>
       <c r="E49" s="85"/>
@@ -39428,7 +39428,7 @@
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B50" s="61" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>40</v>
@@ -39663,7 +39663,7 @@
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B65" s="61" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C65" s="36" t="s">
         <v>40</v>
@@ -39888,7 +39888,7 @@
         <v>27</v>
       </c>
       <c r="C79" s="140" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D79" s="140"/>
       <c r="E79" s="85"/>
@@ -39898,7 +39898,7 @@
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B80" s="61" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C80" s="36" t="s">
         <v>40</v>
@@ -40148,16 +40148,16 @@
     <row r="96" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B96" s="7"/>
       <c r="C96" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="D96" s="22" t="s">
         <v>79</v>
-      </c>
-      <c r="D96" s="22" t="s">
-        <v>80</v>
       </c>
       <c r="E96" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F96" s="22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G96" s="85"/>
       <c r="N96" s="87"/>
@@ -40479,13 +40479,13 @@
     </row>
     <row r="116" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B116" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C116" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E116" s="85"/>
       <c r="F116" s="85"/>
@@ -40494,7 +40494,7 @@
     </row>
     <row r="117" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B117" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C117" s="4">
         <f>'processed | data'!B136</f>
@@ -40572,7 +40572,7 @@
     </row>
     <row r="123" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B123" s="36" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C123" s="36"/>
       <c r="D123" s="36"/>
@@ -40583,7 +40583,7 @@
     </row>
     <row r="124" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B124" s="81" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C124" s="68">
         <f>'processed | data'!B151</f>
@@ -40656,7 +40656,7 @@
     </row>
     <row r="130" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B130" s="82" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C130" s="82">
         <f>SUM(C127:C128)</f>
@@ -40670,7 +40670,7 @@
     </row>
     <row r="131" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B131" s="82" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C131" s="82" t="e">
         <f>ROUND((C130/C107)*100,0)</f>
@@ -40732,7 +40732,7 @@
     </row>
     <row r="136" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B136" s="18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C136" s="11">
         <f>'processed | data'!B157</f>
@@ -40764,10 +40764,10 @@
     </row>
     <row r="139" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B139" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C139" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D139" s="13"/>
       <c r="E139" s="85"/>
@@ -40776,7 +40776,7 @@
     </row>
     <row r="140" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B140" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C140" s="6">
         <f>'processed | data'!B162</f>
@@ -40789,7 +40789,7 @@
     </row>
     <row r="141" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B141" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C141" s="6">
         <f>'processed | data'!B163</f>
@@ -40802,7 +40802,7 @@
     </row>
     <row r="142" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B142" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C142" s="6">
         <f>'processed | data'!B164</f>
@@ -40815,7 +40815,7 @@
     </row>
     <row r="143" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B143" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C143" s="6">
         <f>'processed | data'!B165</f>
@@ -40836,7 +40836,7 @@
     </row>
     <row r="145" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B145" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C145" s="6">
         <f>'processed | data'!B167</f>
@@ -40849,7 +40849,7 @@
     </row>
     <row r="146" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B146" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C146" s="6">
         <f>'processed | data'!B168</f>
@@ -40894,7 +40894,7 @@
     </row>
     <row r="151" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B151" s="95" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C151" s="95" t="s">
         <v>5</v>
@@ -40904,10 +40904,10 @@
       <c r="F151" s="85"/>
       <c r="G151" s="85"/>
       <c r="I151" s="95" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J151" s="95" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="152" spans="2:10" x14ac:dyDescent="0.2">
@@ -41987,12 +41987,12 @@
   <sheetData>
     <row r="1" spans="1:6" s="51" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A1" s="50" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F2" s="8"/>
     </row>
@@ -42005,7 +42005,7 @@
     </row>
     <row r="4" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A4" s="75" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B4" s="75"/>
       <c r="C4" s="75"/>
@@ -42015,21 +42015,21 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="77" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B5" s="77"/>
       <c r="C5"/>
       <c r="D5" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E5" s="72" t="s">
-        <v>120</v>
       </c>
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B6" s="71" cm="1">
         <f t="array" ref="B6">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E6), 0)</f>
@@ -42037,7 +42037,7 @@
       </c>
       <c r="C6"/>
       <c r="D6" s="48" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E6" s="48" t="e">
         <f>MATCH(D6, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42047,7 +42047,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B7" s="71" cm="1">
         <f t="array" ref="B7">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E7), 0)</f>
@@ -42055,7 +42055,7 @@
       </c>
       <c r="C7"/>
       <c r="D7" s="48" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E7" s="48" t="e">
         <f>MATCH(D7, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42065,7 +42065,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B8" s="78" cm="1">
         <f t="array" ref="B8">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E8), 0)</f>
@@ -42073,7 +42073,7 @@
       </c>
       <c r="C8"/>
       <c r="D8" s="48" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E8" s="48" t="e">
         <f>MATCH(D8, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42083,7 +42083,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B9" s="78" cm="1">
         <f t="array" ref="B9">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E9), 0)</f>
@@ -42091,7 +42091,7 @@
       </c>
       <c r="C9"/>
       <c r="D9" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E9" s="48" t="e">
         <f>MATCH(D9, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42136,29 +42136,29 @@
     </row>
     <row r="15" spans="1:6" ht="39.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="75" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B15" s="75"/>
       <c r="C15" s="75"/>
       <c r="D15" s="76" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E15" s="75"/>
       <c r="F15" s="75"/>
     </row>
     <row r="16" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C16" s="49"/>
       <c r="D16" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E16" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E16" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -42347,15 +42347,15 @@
     </row>
     <row r="28" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B28" s="65"/>
       <c r="C28" s="49"/>
       <c r="D28" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E28" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -42544,15 +42544,15 @@
     </row>
     <row r="40" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="35" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B40" s="66"/>
       <c r="C40" s="49"/>
       <c r="D40" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E40" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E40" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -42742,15 +42742,15 @@
     </row>
     <row r="52" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="35" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B52" s="66"/>
       <c r="C52" s="49"/>
       <c r="D52" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E52" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E52" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
@@ -42951,29 +42951,29 @@
     </row>
     <row r="66" spans="1:6" ht="39.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="75" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B66" s="75"/>
       <c r="C66" s="75"/>
       <c r="D66" s="75" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E66" s="75"/>
       <c r="F66" s="75"/>
     </row>
     <row r="67" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C67" s="49"/>
       <c r="D67" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E67" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E67" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
@@ -43162,15 +43162,15 @@
     </row>
     <row r="79" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B79" s="65"/>
       <c r="C79" s="49"/>
       <c r="D79" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E79" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E79" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.2">
@@ -43359,15 +43359,15 @@
     </row>
     <row r="91" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="35" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B91" s="66"/>
       <c r="C91" s="49"/>
       <c r="D91" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E91" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E91" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -43557,15 +43557,15 @@
     </row>
     <row r="103" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="35" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B103" s="66"/>
       <c r="C103" s="49"/>
       <c r="D103" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E103" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E103" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
@@ -43768,14 +43768,14 @@
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B117" s="69"/>
       <c r="D117" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E117" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E117" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.2">
@@ -43787,7 +43787,7 @@
         <v>0</v>
       </c>
       <c r="D118" s="48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E118" s="48" t="e">
         <f>MATCH(D118, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43803,7 +43803,7 @@
         <v>0</v>
       </c>
       <c r="D119" s="48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E119" s="48" t="e">
         <f>MATCH(D119, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43819,7 +43819,7 @@
         <v>0</v>
       </c>
       <c r="D120" s="48" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E120" s="48" t="e">
         <f>MATCH(D120, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43835,7 +43835,7 @@
         <v>0</v>
       </c>
       <c r="D121" s="48" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E121" s="48" t="e">
         <f>MATCH(D121, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43851,7 +43851,7 @@
         <v>0</v>
       </c>
       <c r="D122" s="48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E122" s="48" t="e">
         <f>MATCH(D122, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43874,14 +43874,14 @@
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B126" s="69"/>
       <c r="D126" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E126" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E126" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.2">
@@ -43893,7 +43893,7 @@
         <v>0</v>
       </c>
       <c r="D127" s="48" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E127" s="48" t="e">
         <f>MATCH(D127, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43909,7 +43909,7 @@
         <v>0</v>
       </c>
       <c r="D128" s="48" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E128" s="48" t="e">
         <f>MATCH(D128, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43925,7 +43925,7 @@
         <v>0</v>
       </c>
       <c r="D129" s="48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E129" s="48" t="e">
         <f>MATCH(D129, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43941,7 +43941,7 @@
         <v>0</v>
       </c>
       <c r="D130" s="48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E130" s="48" t="e">
         <f>MATCH(D130, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43957,7 +43957,7 @@
         <v>0</v>
       </c>
       <c r="D131" s="48" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E131" s="48" t="e">
         <f>MATCH(D131, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43980,19 +43980,19 @@
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B135" s="70"/>
       <c r="D135" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E135" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E135" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B136" s="33" cm="1">
         <f t="array" ref="B136">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E136), 0)</f>
@@ -44000,7 +44000,7 @@
       </c>
       <c r="C136"/>
       <c r="D136" s="48" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E136" s="48" t="e">
         <f>MATCH(D136, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44017,7 +44017,7 @@
       </c>
       <c r="C137"/>
       <c r="D137" s="48" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E137" s="48" t="e">
         <f>MATCH(D137, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44034,7 +44034,7 @@
       </c>
       <c r="C138"/>
       <c r="D138" s="48" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E138" s="48" t="e">
         <f>MATCH(D138, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44057,26 +44057,26 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B142" s="70"/>
       <c r="D142" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E142" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E142" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B143" s="33" cm="1">
         <f t="array" ref="B143">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E143), 0)</f>
         <v>0</v>
       </c>
       <c r="D143" s="48" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E143" s="48" t="e">
         <f>MATCH(D143, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44092,7 +44092,7 @@
         <v>0</v>
       </c>
       <c r="D144" s="48" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E144" s="48" t="e">
         <f>MATCH(D144, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44108,7 +44108,7 @@
         <v>0</v>
       </c>
       <c r="D145" s="48" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E145" s="48" t="e">
         <f>MATCH(D145, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44135,7 +44135,7 @@
     </row>
     <row r="149" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A149" s="75" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B149" s="75"/>
       <c r="C149" s="75"/>
@@ -44145,27 +44145,27 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="79" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B150" s="79"/>
       <c r="C150"/>
       <c r="D150" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E150" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E150" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B151" s="80" cm="1">
         <f t="array" ref="B151">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E151), 0)</f>
         <v>0</v>
       </c>
       <c r="D151" s="48" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E151" s="48" t="e">
         <f>MATCH(D151, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44182,14 +44182,14 @@
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B154" s="10"/>
       <c r="D154" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E154" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E154" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.2">
@@ -44201,7 +44201,7 @@
         <v>0</v>
       </c>
       <c r="D155" s="48" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E155" s="48" t="e">
         <f>MATCH(D155, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44217,7 +44217,7 @@
         <v>0</v>
       </c>
       <c r="D156" s="48" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E156" s="48" t="e">
         <f>MATCH(D156, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44227,14 +44227,14 @@
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B157" s="71" cm="1">
         <f t="array" ref="B157">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E157), 0)</f>
         <v>0</v>
       </c>
       <c r="D157" s="48" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E157" s="48" t="e">
         <f>MATCH(D157, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44258,26 +44258,26 @@
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B161" s="69"/>
       <c r="D161" s="72" t="s">
+        <v>118</v>
+      </c>
+      <c r="E161" s="72" t="s">
         <v>119</v>
-      </c>
-      <c r="E161" s="72" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B162" s="38" cm="1">
         <f t="array" ref="B162">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E162), 0)</f>
         <v>0</v>
       </c>
       <c r="D162" s="48" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E162" s="48" t="e">
         <f>MATCH(D162, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44286,14 +44286,14 @@
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B163" s="38">
         <f>B120</f>
         <v>0</v>
       </c>
       <c r="D163" s="48" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E163" s="48" t="e">
         <f>MATCH(D163, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44302,14 +44302,14 @@
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B164" s="38" cm="1">
         <f t="array" ref="B164">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E164), 0)</f>
         <v>0</v>
       </c>
       <c r="D164" s="48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E164" s="48" t="e">
         <f>MATCH(D164, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44318,14 +44318,14 @@
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B165" s="38" cm="1">
         <f t="array" ref="B165">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E165), 0)</f>
         <v>0</v>
       </c>
       <c r="D165" s="48" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E165" s="48" t="e">
         <f>MATCH(D165, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44338,14 +44338,14 @@
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A167" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B167" s="38" cm="1">
         <f t="array" ref="B167">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E167), 0)</f>
         <v>0</v>
       </c>
       <c r="D167" s="48" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E167" s="48" t="e">
         <f>MATCH(D167, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44354,14 +44354,14 @@
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A168" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B168" s="38" cm="1">
         <f t="array" ref="B168">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E168), 0)</f>
         <v>0</v>
       </c>
       <c r="D168" s="48" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E168" s="48" t="e">
         <f>MATCH(D168, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44382,7 +44382,7 @@
     </row>
     <row r="172" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A172" s="75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B172" s="75"/>
       <c r="C172" s="75"/>
@@ -44392,17 +44392,17 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" s="92" t="s">
+        <v>156</v>
+      </c>
+      <c r="B173" s="93" t="s">
         <v>157</v>
-      </c>
-      <c r="B173" s="93" t="s">
-        <v>158</v>
       </c>
       <c r="C173" s="93"/>
       <c r="D173" s="92" t="s">
         <v>5</v>
       </c>
       <c r="E173" s="92" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F173" s="92"/>
     </row>
@@ -48586,23 +48586,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="90" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="90" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="90" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B2" s="91" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="90" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B3" s="96">
         <v>36892</v>
@@ -48610,7 +48610,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="90" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B4" s="96">
         <v>37289</v>
@@ -48618,7 +48618,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="90" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B5" s="91">
         <v>85</v>
@@ -48626,7 +48626,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="90" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B6" s="91">
         <v>66</v>
@@ -48634,7 +48634,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="90" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B7" s="91">
         <v>15.25</v>
@@ -48642,7 +48642,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="90" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B8" s="91">
         <v>15</v>
@@ -48650,7 +48650,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="90" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B9" s="91">
         <v>69.75</v>
@@ -48658,7 +48658,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="90" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B10" s="91">
         <v>51</v>
@@ -48666,7 +48666,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="90" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B11" s="91">
         <v>71</v>
@@ -48674,7 +48674,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="90" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B12" s="91">
         <v>72</v>
@@ -48682,7 +48682,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="90" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B13" s="91">
         <v>11</v>
@@ -48690,7 +48690,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="90" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B14" s="91">
         <v>12</v>
@@ -48698,7 +48698,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="90" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B15" s="91">
         <v>26</v>
@@ -48706,7 +48706,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="90" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B16" s="91">
         <v>33.25</v>
@@ -48714,7 +48714,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="90" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B17" s="91">
         <v>25</v>
@@ -48722,7 +48722,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="90" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B18" s="91">
         <v>36.5</v>
@@ -48730,7 +48730,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="90" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B19" s="91">
         <v>15</v>
@@ -48738,7 +48738,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="90" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B20" s="91">
         <v>15.25</v>
@@ -48746,7 +48746,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="90" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B21" s="91">
         <v>21</v>
@@ -48754,7 +48754,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="90" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B22" s="91">
         <v>23.25</v>
@@ -48762,7 +48762,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="90" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B23" s="91">
         <v>27</v>
@@ -48770,7 +48770,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="90" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B24" s="91">
         <v>35.75</v>
@@ -48778,7 +48778,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="90" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B25" s="91">
         <v>12</v>
@@ -48786,7 +48786,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="90" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B26" s="91">
         <v>15</v>
@@ -48794,7 +48794,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="90" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B27" s="91">
         <v>37</v>
@@ -48802,7 +48802,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="90" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B28" s="91">
         <v>47.25</v>
@@ -48810,7 +48810,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="90" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B29" s="91">
         <v>2</v>
@@ -48818,7 +48818,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="90" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B30" s="91">
         <v>4</v>
@@ -48826,7 +48826,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="90" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B31" s="91">
         <v>7</v>
@@ -48834,7 +48834,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="90" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B32" s="91">
         <v>11</v>
@@ -48842,7 +48842,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="90" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B33" s="91">
         <v>2</v>
@@ -48850,7 +48850,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="90" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B34" s="91">
         <v>4</v>
@@ -48858,7 +48858,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="90" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B35" s="91">
         <v>1</v>
@@ -48866,7 +48866,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="90" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B36" s="91">
         <v>5</v>
@@ -48874,7 +48874,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="90" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B37" s="91">
         <v>1</v>
@@ -48882,7 +48882,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="90" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B38" s="91">
         <v>0.5</v>
@@ -48890,7 +48890,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="90" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B39" s="91">
         <v>4</v>
@@ -48898,7 +48898,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="90" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B40" s="91">
         <v>1.25</v>
@@ -48906,7 +48906,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="90" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B41" s="91">
         <v>3</v>
@@ -48914,7 +48914,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="90" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B42" s="91">
         <v>1</v>
@@ -48922,7 +48922,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="90" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B43" s="91">
         <v>1</v>
@@ -48930,7 +48930,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="90" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B44" s="91">
         <v>0.25</v>
@@ -48938,7 +48938,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="90" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B45" s="91">
         <v>1</v>
@@ -48946,7 +48946,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="90" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B46" s="91">
         <v>0.25</v>
@@ -48954,7 +48954,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="90" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B47" s="91">
         <v>26</v>
@@ -48962,7 +48962,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="90" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B48" s="91">
         <v>31.5</v>
@@ -48970,7 +48970,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="90" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B49" s="91">
         <v>15</v>
@@ -48978,7 +48978,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="90" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B50" s="91">
         <v>25</v>
@@ -48986,7 +48986,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="90" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B51" s="91">
         <v>25</v>
@@ -48994,7 +48994,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="90" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B52" s="91">
         <v>28.5</v>
@@ -49002,7 +49002,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="90" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B53" s="91">
         <v>2</v>
@@ -49010,7 +49010,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="90" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B54" s="91">
         <v>0</v>
@@ -49018,7 +49018,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="90" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B55" s="91">
         <v>6</v>
@@ -49026,7 +49026,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="90" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B56" s="91">
         <v>7.25</v>
@@ -49034,7 +49034,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="90" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B57" s="91">
         <v>9</v>
@@ -49042,7 +49042,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="90" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B58" s="91">
         <v>12.5</v>
@@ -49050,7 +49050,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" s="90" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B59" s="91">
         <v>2</v>
@@ -49058,7 +49058,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" s="90" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B60" s="91">
         <v>2.5</v>
@@ -49066,7 +49066,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="90" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B61" s="91">
         <v>1</v>
@@ -49074,7 +49074,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="90" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B62" s="91">
         <v>2</v>
@@ -49082,7 +49082,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="90" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B63" s="91">
         <v>4</v>
@@ -49090,7 +49090,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="90" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B64" s="91">
         <v>4.5</v>
@@ -49098,7 +49098,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="90" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B65" s="91">
         <v>1</v>
@@ -49106,7 +49106,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="90" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B66" s="91">
         <v>1</v>
@@ -49114,7 +49114,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="90" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B67" s="91">
         <v>3</v>
@@ -49122,7 +49122,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="90" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B68" s="91">
         <v>0.25</v>
@@ -49130,7 +49130,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="90" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B69" s="91">
         <v>2</v>
@@ -49138,7 +49138,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="90" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B70" s="91">
         <v>0</v>
@@ -49146,7 +49146,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="90" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B71" s="91">
         <v>1</v>
@@ -49154,7 +49154,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="90" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B72" s="91">
         <v>0.25</v>
@@ -49162,7 +49162,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="90" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B73" s="91">
         <v>1</v>
@@ -49170,7 +49170,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" s="90" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B74" s="91">
         <v>0.25</v>
@@ -49178,7 +49178,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" s="90" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B75" s="91">
         <v>10</v>
@@ -49186,7 +49186,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" s="90" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B76" s="91">
         <v>13</v>
@@ -49194,7 +49194,7 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" s="90" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B77" s="91">
         <v>5</v>
@@ -49202,7 +49202,7 @@
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" s="90" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B78" s="91">
         <v>2.25</v>
@@ -49210,7 +49210,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" s="90" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B79" s="91">
         <v>2</v>
@@ -49218,7 +49218,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" s="90" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B80" s="91">
         <v>2.75</v>
@@ -49226,7 +49226,7 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" s="90" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B81" s="91">
         <v>2</v>
@@ -49234,7 +49234,7 @@
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" s="90" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B82" s="91">
         <v>2</v>
@@ -49242,7 +49242,7 @@
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" s="90" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B83" s="91">
         <v>4</v>
@@ -49250,7 +49250,7 @@
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" s="90" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B84" s="91">
         <v>4.5</v>
@@ -49258,7 +49258,7 @@
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" s="90" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B85" s="91">
         <v>1</v>
@@ -49266,7 +49266,7 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" s="90" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B86" s="91">
         <v>0</v>
@@ -49274,7 +49274,7 @@
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" s="90" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B87" s="91">
         <v>2</v>
@@ -49282,7 +49282,7 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" s="90" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B88" s="91">
         <v>2.5</v>
@@ -49290,7 +49290,7 @@
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" s="90" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B89" s="91">
         <v>2</v>
@@ -49298,7 +49298,7 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" s="90" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B90" s="91">
         <v>3</v>
@@ -49306,7 +49306,7 @@
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" s="90" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B91" s="91">
         <v>5</v>
@@ -49314,7 +49314,7 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="90" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B92" s="91">
         <v>3.75</v>
@@ -49322,7 +49322,7 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="90" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B93" s="91">
         <v>4</v>
@@ -49330,7 +49330,7 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="90" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B94" s="91">
         <v>5.5</v>
@@ -49338,7 +49338,7 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="90" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B95" s="91">
         <v>2</v>
@@ -49346,7 +49346,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="90" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B96" s="91">
         <v>0</v>
@@ -49354,7 +49354,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="90" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B97" s="91">
         <v>1</v>
@@ -49362,7 +49362,7 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" s="90" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B98" s="91">
         <v>3</v>
@@ -49370,7 +49370,7 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" s="90" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B99" s="91">
         <v>1</v>
@@ -49378,7 +49378,7 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" s="90" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B100" s="91">
         <v>0.5</v>
@@ -49386,7 +49386,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" s="90" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B101" s="91">
         <v>2</v>
@@ -49394,7 +49394,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" s="90" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B102" s="91">
         <v>2.5</v>
@@ -49402,7 +49402,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" s="90" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B103" s="91">
         <v>1</v>
@@ -49410,7 +49410,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" s="90" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B104" s="91">
         <v>0.5</v>
@@ -49418,7 +49418,7 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" s="90" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B105" s="91">
         <v>1</v>
@@ -49426,7 +49426,7 @@
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" s="90" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B106" s="91">
         <v>1</v>
@@ -49434,7 +49434,7 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" s="90" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B107" s="91">
         <v>4</v>
@@ -49442,7 +49442,7 @@
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" s="90" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B108" s="91">
         <v>10</v>
@@ -49450,7 +49450,7 @@
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" s="90" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B109" s="91">
         <v>5</v>
@@ -49458,7 +49458,7 @@
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" s="90" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B110" s="91">
         <v>8</v>
@@ -49466,7 +49466,7 @@
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" s="90" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B111" s="91">
         <v>2</v>
@@ -49474,7 +49474,7 @@
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" s="90" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B112" s="91">
         <v>3</v>
@@ -49482,7 +49482,7 @@
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" s="90" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B113" s="91">
         <v>2</v>
@@ -49490,7 +49490,7 @@
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" s="90" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B114" s="91">
         <v>5</v>
@@ -49498,7 +49498,7 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" s="90" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B115" s="91">
         <v>6</v>
@@ -49506,7 +49506,7 @@
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" s="90" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B116" s="91">
         <v>7.5</v>
@@ -49514,7 +49514,7 @@
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" s="90" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B117" s="91">
         <v>5</v>
@@ -49522,7 +49522,7 @@
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="90" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B118" s="91">
         <v>6</v>
@@ -49530,7 +49530,7 @@
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" s="90" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B119" s="91">
         <v>5</v>
@@ -49538,7 +49538,7 @@
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" s="90" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B120" s="91">
         <v>6.5</v>
@@ -49546,7 +49546,7 @@
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" s="90" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B121" s="91">
         <v>1</v>
@@ -49554,7 +49554,7 @@
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" s="90" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B122" s="91">
         <v>0.5</v>
@@ -49562,7 +49562,7 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" s="90" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B123" s="91">
         <v>1</v>
@@ -49570,7 +49570,7 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" s="90" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B124" s="91">
         <v>1</v>
@@ -49578,7 +49578,7 @@
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" s="90" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B125" s="91">
         <v>1</v>
@@ -49586,7 +49586,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" s="90" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B126" s="91">
         <v>3</v>
@@ -49594,7 +49594,7 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" s="90" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B127" s="91">
         <v>3</v>
@@ -49602,7 +49602,7 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" s="90" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B128" s="91">
         <v>1</v>
@@ -49610,7 +49610,7 @@
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" s="90" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B129" s="91">
         <v>1</v>
@@ -49618,7 +49618,7 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" s="90" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B130" s="91">
         <v>2</v>
@@ -49626,7 +49626,7 @@
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" s="90" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B131" s="91">
         <v>14</v>
@@ -49634,7 +49634,7 @@
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" s="90" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B132" s="91">
         <v>19</v>
@@ -49642,7 +49642,7 @@
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A133" s="90" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B133" s="91">
         <v>1.3</v>
@@ -49650,7 +49650,7 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A134" s="90" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B134" s="91">
         <v>7</v>
@@ -49658,7 +49658,7 @@
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A135" s="90" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B135" s="91">
         <v>11</v>
@@ -49666,7 +49666,7 @@
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A136" s="90" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B136" s="91">
         <v>30</v>
@@ -49674,7 +49674,7 @@
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A137" s="90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B137" s="91">
         <v>40</v>
@@ -49682,7 +49682,7 @@
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" s="90" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B138" s="91">
         <v>40</v>
@@ -49690,7 +49690,7 @@
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A139" s="90" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B139" s="91">
         <v>45</v>
@@ -49698,7 +49698,7 @@
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" s="90" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B140" s="91">
         <v>45</v>
@@ -49706,7 +49706,7 @@
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A141" s="90" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B141" s="91" t="b">
         <v>0</v>
@@ -49714,7 +49714,7 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" s="90" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B142" s="91" t="b">
         <v>0</v>
@@ -49722,7 +49722,7 @@
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A143" s="90" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B143" s="91" t="b">
         <v>0</v>
@@ -49730,7 +49730,7 @@
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A144" s="90" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B144" s="91" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Fix: excel template | Improve description for calculated stats tab optional metadata config
</commit_message>
<xml_diff>
--- a/assets/xlsx/visualise-metrics.xlsx
+++ b/assets/xlsx/visualise-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christracey/workspace/sprint-metrics_webapp/assets/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D58F707-7C17-8D43-BDAF-1D9A348601BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50AF3DA0-69CC-AF42-A7E9-46914B8A1452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="783" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,9 +488,6 @@
     <t>estimate</t>
   </si>
   <si>
-    <t>Configure the labels you are interested in here only</t>
-  </si>
-  <si>
     <t>DON’T EDIT THIS LIST (USE CONFIG ABOVE)</t>
   </si>
   <si>
@@ -555,12 +552,6 @@
   </si>
   <si>
     <t>component3</t>
-  </si>
-  <si>
-    <t>label1</t>
-  </si>
-  <si>
-    <t>label2</t>
   </si>
   <si>
     <t>Parents</t>
@@ -982,12 +973,23 @@
   <si>
     <t>committed at sprint start (+)</t>
   </si>
+  <si>
+    <t>[Optional] Configure the metadata for meta data template.
+List below the labels and components you need to report on.
+(DON’T Edit BAU/Improvement labels)</t>
+  </si>
+  <si>
+    <t>label3</t>
+  </si>
+  <si>
+    <t>label4</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1169,6 +1171,13 @@
       <b/>
       <sz val="10"/>
       <color theme="1" tint="0.34998626667073579"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4" tint="0.39997558519241921"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1662,7 +1671,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1944,6 +1953,10 @@
     <xf numFmtId="0" fontId="2" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
@@ -3975,10 +3988,10 @@
                   <c:v>BAU/Improvement</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>label1</c:v>
+                  <c:v>label3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>label2</c:v>
+                  <c:v>label4</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -19322,129 +19335,6 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>562595</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>37376</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>2439</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>221523</xdr:rowOff>
-    </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="18" name="Group 17">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5488E59E-8FC1-0242-BDB6-FFE1D562E95F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
-        <a:xfrm>
-          <a:off x="1349995" y="7314476"/>
-          <a:ext cx="5688244" cy="2025647"/>
-          <a:chOff x="1164168" y="6272568"/>
-          <a:chExt cx="5556249" cy="1838113"/>
-        </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="19" name="Picture 18">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3FFC5E38-82E4-D71F-3757-81AE43F2FF86}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill rotWithShape="1">
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect b="4428"/>
-          <a:stretch/>
-        </xdr:blipFill>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="1164168" y="6272568"/>
-            <a:ext cx="5556249" cy="1838113"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="20" name="TextBox 19">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7B6F0A0-A728-EF42-0650-5883B4279BF2}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr txBox="1"/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm rot="20758441">
-            <a:off x="1731086" y="6809981"/>
-            <a:ext cx="3966584" cy="797820"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln w="9525" cmpd="sng">
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:lnRef>
-          <a:fillRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="dk1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:r>
-              <a:rPr lang="en-GB" sz="6600">
-                <a:solidFill>
-                  <a:srgbClr val="EA9191"/>
-                </a:solidFill>
-                <a:latin typeface="Stencil" pitchFamily="82" charset="77"/>
-              </a:rPr>
-              <a:t>SAMPLE</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-    </xdr:grpSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
       <xdr:colOff>62659</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>515258</xdr:rowOff>
@@ -19474,7 +19364,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -19512,7 +19402,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -23845,7 +23735,7 @@
         </xdr:xfrm>
         <a:graphic>
           <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
           </a:graphicData>
         </a:graphic>
       </xdr:graphicFrame>
@@ -23868,7 +23758,7 @@
         </xdr:xfrm>
         <a:graphic>
           <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           </a:graphicData>
         </a:graphic>
       </xdr:graphicFrame>
@@ -23942,7 +23832,7 @@
         </xdr:xfrm>
         <a:graphic>
           <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+            <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
           </a:graphicData>
         </a:graphic>
       </xdr:graphicFrame>
@@ -24845,13 +24735,13 @@
           </xdr:cNvPicPr>
         </xdr:nvPicPr>
         <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8">
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
             <a:extLst>
               <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
                 <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
               </a:ext>
               <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId9"/>
+                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId8"/>
               </a:ext>
             </a:extLst>
           </a:blip>
@@ -24883,13 +24773,13 @@
           </xdr:cNvPicPr>
         </xdr:nvPicPr>
         <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10">
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
             <a:extLst>
               <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
                 <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
               </a:ext>
               <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId11"/>
+                <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId10"/>
               </a:ext>
             </a:extLst>
           </a:blip>
@@ -24972,6 +24862,129 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Calibri"/>
             </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>939800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2668819</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>222247</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="119" name="Group 118">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D901158-3EF1-6249-94F8-8029FFC285F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="1143000" y="7035800"/>
+          <a:ext cx="5424719" cy="2025647"/>
+          <a:chOff x="1164168" y="6272568"/>
+          <a:chExt cx="5556249" cy="1838113"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="120" name="Picture 119">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5D05110C-C78B-79D2-64D1-530CA7AD35DC}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill rotWithShape="1">
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:srcRect b="4428"/>
+          <a:stretch/>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1164168" y="6272568"/>
+            <a:ext cx="5556249" cy="1838113"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="121" name="TextBox 120">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FEEB407-052D-5B28-F72D-E7CAFA0CE51B}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="20758441">
+            <a:off x="1688931" y="6815105"/>
+            <a:ext cx="4009377" cy="797820"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="9525" cmpd="sng">
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-GB" sz="6600">
+                <a:solidFill>
+                  <a:srgbClr val="EA9191"/>
+                </a:solidFill>
+                <a:latin typeface="Stencil" pitchFamily="82" charset="77"/>
+              </a:rPr>
+              <a:t>SAMPLE</a:t>
+            </a:r>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -25957,14 +25970,14 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>562595</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>37376</xdr:rowOff>
+      <xdr:colOff>359395</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>939076</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>2875814</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:colOff>2672614</xdr:colOff>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>221523</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
@@ -25980,7 +25993,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1349995" y="7314476"/>
+          <a:off x="1146795" y="7035076"/>
           <a:ext cx="5424719" cy="2025647"/>
           <a:chOff x="1164168" y="6272568"/>
           <a:chExt cx="5556249" cy="1838113"/>
@@ -28273,7 +28286,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="14015005" y="5918697"/>
+              <a:off x="14015005" y="5904593"/>
               <a:ext cx="1211676" cy="588956"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -28341,7 +28354,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="15245705" y="5933266"/>
+              <a:off x="15245705" y="5919162"/>
               <a:ext cx="1198273" cy="589336"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -28409,7 +28422,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="16440288" y="5936717"/>
+              <a:off x="16440288" y="5922612"/>
               <a:ext cx="1156607" cy="589336"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -29256,8 +29269,8 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="5400000" flipH="1" flipV="1">
-              <a:off x="14813791" y="4890959"/>
-              <a:ext cx="834789" cy="1220686"/>
+              <a:off x="14820844" y="4883908"/>
+              <a:ext cx="820686" cy="1220686"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
               <a:avLst>
@@ -29299,8 +29312,8 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="16200000" flipV="1">
-              <a:off x="15418507" y="5506931"/>
-              <a:ext cx="849359" cy="3312"/>
+              <a:off x="15425559" y="5499879"/>
+              <a:ext cx="835254" cy="3312"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
               <a:avLst>
@@ -29342,8 +29355,8 @@
           </xdr:nvCxnSpPr>
           <xdr:spPr>
             <a:xfrm rot="16200000" flipH="1">
-              <a:off x="16003656" y="4921781"/>
-              <a:ext cx="852809" cy="1177063"/>
+              <a:off x="16010709" y="4914728"/>
+              <a:ext cx="838705" cy="1177063"/>
             </a:xfrm>
             <a:prstGeom prst="curvedConnector3">
               <a:avLst>
@@ -32403,7 +32416,7 @@
                     <a:cs typeface="Calibri"/>
                   </a:rPr>
                   <a:pPr algn="r"/>
-                  <a:t>label1</a:t>
+                  <a:t>label3</a:t>
                 </a:fld>
                 <a:endParaRPr lang="en-AU" sz="800">
                   <a:solidFill>
@@ -32717,7 +32730,7 @@
                     <a:cs typeface="Calibri"/>
                   </a:rPr>
                   <a:pPr algn="r"/>
-                  <a:t>label2</a:t>
+                  <a:t>label4</a:t>
                 </a:fld>
                 <a:endParaRPr lang="en-AU" sz="800">
                   <a:solidFill>
@@ -36765,11 +36778,11 @@
       <c r="G8" s="104"/>
       <c r="H8" s="105"/>
       <c r="I8" s="133" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="J8" s="133"/>
       <c r="K8" s="133" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="L8" s="133"/>
       <c r="M8" s="106"/>
@@ -36876,7 +36889,7 @@
       <c r="F12" s="132"/>
       <c r="G12" s="104"/>
       <c r="H12" s="113" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="I12" s="116">
         <f>'Sprint Summary | data'!R21</f>
@@ -37202,11 +37215,11 @@
       <c r="G8" s="104"/>
       <c r="H8" s="105"/>
       <c r="I8" s="133" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="J8" s="133"/>
       <c r="K8" s="133" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="L8" s="133"/>
       <c r="M8" s="106"/>
@@ -37313,7 +37326,7 @@
       <c r="F12" s="132"/>
       <c r="G12" s="104"/>
       <c r="H12" s="113" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="I12" s="116">
         <f>'Sprint Summary | data'!R21</f>
@@ -37564,7 +37577,7 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B5" s="4">
         <f>'Calculated Stats'!C22</f>
@@ -38202,7 +38215,7 @@
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>label1</v>
+        <v>label3</v>
       </c>
       <c r="B30" s="34">
         <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A30, 'Calculated Stats'!B$36:B$45, 0))</f>
@@ -38234,7 +38247,7 @@
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>label2</v>
+        <v>label4</v>
       </c>
       <c r="B31" s="34">
         <f>INDEX('Calculated Stats'!D$36:D$45, MATCH(A31, 'Calculated Stats'!B$36:B$45, 0))</f>
@@ -38885,9 +38898,9 @@
       <c r="F5" s="86"/>
       <c r="G5" s="85"/>
     </row>
-    <row r="6" spans="2:7" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="134" t="s">
-        <v>130</v>
+    <row r="6" spans="2:7" ht="63" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="141" t="s">
+        <v>278</v>
       </c>
       <c r="C6" s="135"/>
       <c r="D6" s="85"/>
@@ -38908,11 +38921,11 @@
       <c r="G7" s="85"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="142" t="s">
         <v>1</v>
       </c>
       <c r="C8" s="59" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D8" s="85"/>
       <c r="E8" s="85"/>
@@ -38920,11 +38933,11 @@
       <c r="G8" s="85"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="142" t="s">
         <v>53</v>
       </c>
       <c r="C9" s="59" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D9" s="85"/>
       <c r="E9" s="85"/>
@@ -38933,10 +38946,10 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="56" t="s">
-        <v>153</v>
+        <v>279</v>
       </c>
       <c r="C10" s="59" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D10" s="85"/>
       <c r="E10" s="85"/>
@@ -38945,7 +38958,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="56" t="s">
-        <v>154</v>
+        <v>280</v>
       </c>
       <c r="C11" s="59"/>
       <c r="D11" s="85"/>
@@ -39043,7 +39056,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="77" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C20" s="77"/>
       <c r="D20" s="85"/>
@@ -39053,7 +39066,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C21" s="11">
         <f>'processed | data'!B6</f>
@@ -39066,7 +39079,7 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C22" s="11">
         <f>'processed | data'!B7</f>
@@ -39079,7 +39092,7 @@
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C23" s="11" t="str">
         <f>TEXT('processed | data'!B8, "DD/MM/YYYY")</f>
@@ -39092,7 +39105,7 @@
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C24" s="11" t="str">
         <f>TEXT('processed | data'!B9, "DD/MM/YYYY")</f>
@@ -39161,7 +39174,7 @@
     </row>
     <row r="32" spans="2:7" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="134" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C32" s="135"/>
       <c r="D32" s="28"/>
@@ -39193,7 +39206,7 @@
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B35" s="61" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C35" s="52" t="s">
         <v>40</v>
@@ -39245,7 +39258,7 @@
     <row r="38" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B38" s="62" t="str">
         <f t="shared" si="0"/>
-        <v>label1</v>
+        <v>label3</v>
       </c>
       <c r="C38" s="4">
         <f>'processed | data'!B19</f>
@@ -39263,7 +39276,7 @@
     <row r="39" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B39" s="62" t="str">
         <f t="shared" si="0"/>
-        <v>label2</v>
+        <v>label4</v>
       </c>
       <c r="C39" s="4">
         <f>'processed | data'!B20</f>
@@ -39428,7 +39441,7 @@
     </row>
     <row r="50" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B50" s="61" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>40</v>
@@ -39480,7 +39493,7 @@
     <row r="53" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B53" s="62" t="str">
         <f t="shared" si="1"/>
-        <v>label1</v>
+        <v>label3</v>
       </c>
       <c r="C53" s="4">
         <f>'processed | data'!B70</f>
@@ -39498,7 +39511,7 @@
     <row r="54" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B54" s="62" t="str">
         <f t="shared" si="1"/>
-        <v>label2</v>
+        <v>label4</v>
       </c>
       <c r="C54" s="4">
         <f>'processed | data'!B71</f>
@@ -39663,7 +39676,7 @@
     </row>
     <row r="65" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B65" s="61" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C65" s="36" t="s">
         <v>40</v>
@@ -39898,7 +39911,7 @@
     </row>
     <row r="80" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B80" s="61" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C80" s="36" t="s">
         <v>40</v>
@@ -40572,7 +40585,7 @@
     </row>
     <row r="123" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B123" s="36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C123" s="36"/>
       <c r="D123" s="36"/>
@@ -40583,7 +40596,7 @@
     </row>
     <row r="124" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B124" s="81" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C124" s="68">
         <f>'processed | data'!B151</f>
@@ -40670,7 +40683,7 @@
     </row>
     <row r="131" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B131" s="82" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C131" s="82" t="e">
         <f>ROUND((C130/C107)*100,0)</f>
@@ -40732,7 +40745,7 @@
     </row>
     <row r="136" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B136" s="18" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C136" s="11">
         <f>'processed | data'!B157</f>
@@ -40894,7 +40907,7 @@
     </row>
     <row r="151" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B151" s="95" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C151" s="95" t="s">
         <v>5</v>
@@ -40904,10 +40917,10 @@
       <c r="F151" s="85"/>
       <c r="G151" s="85"/>
       <c r="I151" s="95" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="J151" s="95" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="152" spans="2:10" x14ac:dyDescent="0.2">
@@ -41992,7 +42005,7 @@
     </row>
     <row r="2" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F2" s="8"/>
     </row>
@@ -42005,7 +42018,7 @@
     </row>
     <row r="4" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A4" s="75" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B4" s="75"/>
       <c r="C4" s="75"/>
@@ -42015,7 +42028,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="77" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B5" s="77"/>
       <c r="C5"/>
@@ -42029,7 +42042,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B6" s="71" cm="1">
         <f t="array" ref="B6">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E6), 0)</f>
@@ -42047,7 +42060,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B7" s="71" cm="1">
         <f t="array" ref="B7">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E7), 0)</f>
@@ -42065,7 +42078,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B8" s="78" cm="1">
         <f t="array" ref="B8">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E8), 0)</f>
@@ -42083,7 +42096,7 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B9" s="78" cm="1">
         <f t="array" ref="B9">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E9), 0)</f>
@@ -42136,12 +42149,12 @@
     </row>
     <row r="15" spans="1:6" ht="39.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="75" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B15" s="75"/>
       <c r="C15" s="75"/>
       <c r="D15" s="76" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E15" s="75"/>
       <c r="F15" s="75"/>
@@ -42200,7 +42213,7 @@
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="64" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>label1</v>
+        <v>label3</v>
       </c>
       <c r="B19" s="33" cm="1">
         <f t="array" ref="B19">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E19), 0)</f>
@@ -42208,7 +42221,7 @@
       </c>
       <c r="D19" s="48" t="str">
         <f>_xlfn.CONCAT("labels_", A19,"_",D$15)</f>
-        <v>labels_label1_storyPoints</v>
+        <v>labels_label3_storyPoints</v>
       </c>
       <c r="E19" s="48" t="e">
         <f>MATCH(D19, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42218,7 +42231,7 @@
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="64" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>label2</v>
+        <v>label4</v>
       </c>
       <c r="B20" s="33" cm="1">
         <f t="array" ref="B20">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E20), 0)</f>
@@ -42226,7 +42239,7 @@
       </c>
       <c r="D20" s="48" t="str">
         <f>_xlfn.CONCAT("labels_", A20, "_",D$15)</f>
-        <v>labels_label2_storyPoints</v>
+        <v>labels_label4_storyPoints</v>
       </c>
       <c r="E20" s="48" t="e">
         <f>MATCH(D20, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42397,7 +42410,7 @@
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="64" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>label1</v>
+        <v>label3</v>
       </c>
       <c r="B31" s="33" cm="1">
         <f t="array" ref="B31">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E31), 0)</f>
@@ -42405,7 +42418,7 @@
       </c>
       <c r="D31" s="48" t="str">
         <f t="shared" si="0"/>
-        <v>completedLabels_label1_storyPoints</v>
+        <v>completedLabels_label3_storyPoints</v>
       </c>
       <c r="E31" s="48" t="e">
         <f>MATCH(D31, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42415,7 +42428,7 @@
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="64" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>label2</v>
+        <v>label4</v>
       </c>
       <c r="B32" s="33" cm="1">
         <f t="array" ref="B32">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E32), 0)</f>
@@ -42423,7 +42436,7 @@
       </c>
       <c r="D32" s="48" t="str">
         <f t="shared" si="0"/>
-        <v>completedLabels_label2_storyPoints</v>
+        <v>completedLabels_label4_storyPoints</v>
       </c>
       <c r="E32" s="48" t="e">
         <f>MATCH(D32, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -42742,7 +42755,7 @@
     </row>
     <row r="52" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B52" s="66"/>
       <c r="C52" s="49"/>
@@ -42951,12 +42964,12 @@
     </row>
     <row r="66" spans="1:6" ht="39.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="75" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B66" s="75"/>
       <c r="C66" s="75"/>
       <c r="D66" s="75" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E66" s="75"/>
       <c r="F66" s="75"/>
@@ -43015,7 +43028,7 @@
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="64" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>label1</v>
+        <v>label3</v>
       </c>
       <c r="B70" s="33" cm="1">
         <f t="array" ref="B70">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E70), 0)</f>
@@ -43023,7 +43036,7 @@
       </c>
       <c r="D70" s="48" t="str">
         <f>_xlfn.CONCAT("labels_", A70,"_",D$66)</f>
-        <v>labels_label1_count</v>
+        <v>labels_label3_count</v>
       </c>
       <c r="E70" s="48" t="e">
         <f>MATCH(D70, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43033,7 +43046,7 @@
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="64" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>label2</v>
+        <v>label4</v>
       </c>
       <c r="B71" s="33" cm="1">
         <f t="array" ref="B71">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E71), 0)</f>
@@ -43041,7 +43054,7 @@
       </c>
       <c r="D71" s="48" t="str">
         <f>_xlfn.CONCAT("labels_", A71, "_",D$66)</f>
-        <v>labels_label2_count</v>
+        <v>labels_label4_count</v>
       </c>
       <c r="E71" s="48" t="e">
         <f>MATCH(D71, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43212,7 +43225,7 @@
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="64" t="str">
         <f>'Calculated Stats'!B10</f>
-        <v>label1</v>
+        <v>label3</v>
       </c>
       <c r="B82" s="33" cm="1">
         <f t="array" ref="B82">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E82), 0)</f>
@@ -43220,7 +43233,7 @@
       </c>
       <c r="D82" s="48" t="str">
         <f t="shared" si="3"/>
-        <v>completedLabels_label1_count</v>
+        <v>completedLabels_label3_count</v>
       </c>
       <c r="E82" s="48" t="e">
         <f>MATCH(D82, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43230,7 +43243,7 @@
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="64" t="str">
         <f>'Calculated Stats'!B11</f>
-        <v>label2</v>
+        <v>label4</v>
       </c>
       <c r="B83" s="33" cm="1">
         <f t="array" ref="B83">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E83), 0)</f>
@@ -43238,7 +43251,7 @@
       </c>
       <c r="D83" s="48" t="str">
         <f t="shared" si="3"/>
-        <v>completedLabels_label2_count</v>
+        <v>completedLabels_label4_count</v>
       </c>
       <c r="E83" s="48" t="e">
         <f>MATCH(D83, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -43557,7 +43570,7 @@
     </row>
     <row r="103" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="35" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B103" s="66"/>
       <c r="C103" s="49"/>
@@ -44135,7 +44148,7 @@
     </row>
     <row r="149" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A149" s="75" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B149" s="75"/>
       <c r="C149" s="75"/>
@@ -44145,7 +44158,7 @@
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="79" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B150" s="79"/>
       <c r="C150"/>
@@ -44158,7 +44171,7 @@
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B151" s="80" cm="1">
         <f t="array" ref="B151">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E151), 0)</f>
@@ -44227,14 +44240,14 @@
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="18" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B157" s="71" cm="1">
         <f t="array" ref="B157">IFERROR(INDEX('rawdata | iteration analysis'!$2:$2, E157), 0)</f>
         <v>0</v>
       </c>
       <c r="D157" s="48" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E157" s="48" t="e">
         <f>MATCH(D157, 'rawdata | iteration analysis'!$1:$1, )</f>
@@ -44382,7 +44395,7 @@
     </row>
     <row r="172" spans="1:6" ht="26" x14ac:dyDescent="0.2">
       <c r="A172" s="75" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B172" s="75"/>
       <c r="C172" s="75"/>
@@ -44392,17 +44405,17 @@
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" s="92" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B173" s="93" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C173" s="93"/>
       <c r="D173" s="92" t="s">
         <v>5</v>
       </c>
       <c r="E173" s="92" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F173" s="92"/>
     </row>
@@ -48589,7 +48602,7 @@
         <v>87</v>
       </c>
       <c r="B1" s="90" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -48597,7 +48610,7 @@
         <v>88</v>
       </c>
       <c r="B2" s="91" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -48746,7 +48759,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="90" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B21" s="91">
         <v>21</v>
@@ -48754,7 +48767,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="90" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B22" s="91">
         <v>23.25</v>
@@ -48762,7 +48775,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="90" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B23" s="91">
         <v>27</v>
@@ -48770,7 +48783,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="90" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B24" s="91">
         <v>35.75</v>
@@ -48778,7 +48791,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="90" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B25" s="91">
         <v>12</v>
@@ -48786,7 +48799,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" s="90" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B26" s="91">
         <v>15</v>
@@ -48794,7 +48807,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" s="90" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B27" s="91">
         <v>37</v>
@@ -48802,7 +48815,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="90" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B28" s="91">
         <v>47.25</v>
@@ -48810,7 +48823,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" s="90" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B29" s="91">
         <v>2</v>
@@ -48818,7 +48831,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" s="90" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B30" s="91">
         <v>4</v>
@@ -48826,7 +48839,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" s="90" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B31" s="91">
         <v>7</v>
@@ -48834,7 +48847,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="90" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B32" s="91">
         <v>11</v>
@@ -48842,7 +48855,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" s="90" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B33" s="91">
         <v>2</v>
@@ -48850,7 +48863,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" s="90" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B34" s="91">
         <v>4</v>
@@ -48858,7 +48871,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" s="90" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B35" s="91">
         <v>1</v>
@@ -48866,7 +48879,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" s="90" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B36" s="91">
         <v>5</v>
@@ -48874,7 +48887,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" s="90" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B37" s="91">
         <v>1</v>
@@ -48882,7 +48895,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" s="90" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B38" s="91">
         <v>0.5</v>
@@ -48890,7 +48903,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" s="90" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B39" s="91">
         <v>4</v>
@@ -48898,7 +48911,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="90" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B40" s="91">
         <v>1.25</v>
@@ -48906,7 +48919,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" s="90" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B41" s="91">
         <v>3</v>
@@ -48914,7 +48927,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" s="90" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B42" s="91">
         <v>1</v>
@@ -48922,7 +48935,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" s="90" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B43" s="91">
         <v>1</v>
@@ -48930,7 +48943,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" s="90" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B44" s="91">
         <v>0.25</v>
@@ -48938,7 +48951,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" s="90" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B45" s="91">
         <v>1</v>
@@ -48946,7 +48959,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" s="90" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B46" s="91">
         <v>0.25</v>
@@ -48954,7 +48967,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" s="90" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B47" s="91">
         <v>26</v>
@@ -48962,7 +48975,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" s="90" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B48" s="91">
         <v>31.5</v>
@@ -48970,7 +48983,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="90" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B49" s="91">
         <v>15</v>
@@ -48978,7 +48991,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="90" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B50" s="91">
         <v>25</v>
@@ -48986,7 +48999,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="90" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B51" s="91">
         <v>25</v>
@@ -48994,7 +49007,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="90" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B52" s="91">
         <v>28.5</v>
@@ -49002,7 +49015,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="90" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B53" s="91">
         <v>2</v>
@@ -49010,7 +49023,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="90" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B54" s="91">
         <v>0</v>
@@ -49018,7 +49031,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="90" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B55" s="91">
         <v>6</v>
@@ -49026,7 +49039,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="90" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B56" s="91">
         <v>7.25</v>
@@ -49034,7 +49047,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="90" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B57" s="91">
         <v>9</v>
@@ -49042,7 +49055,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="90" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B58" s="91">
         <v>12.5</v>
@@ -49050,7 +49063,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" s="90" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B59" s="91">
         <v>2</v>
@@ -49058,7 +49071,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" s="90" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B60" s="91">
         <v>2.5</v>
@@ -49066,7 +49079,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" s="90" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B61" s="91">
         <v>1</v>
@@ -49074,7 +49087,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" s="90" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B62" s="91">
         <v>2</v>
@@ -49082,7 +49095,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" s="90" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B63" s="91">
         <v>4</v>
@@ -49090,7 +49103,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" s="90" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B64" s="91">
         <v>4.5</v>
@@ -49098,7 +49111,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" s="90" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B65" s="91">
         <v>1</v>
@@ -49106,7 +49119,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" s="90" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B66" s="91">
         <v>1</v>
@@ -49114,7 +49127,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" s="90" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B67" s="91">
         <v>3</v>
@@ -49122,7 +49135,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" s="90" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B68" s="91">
         <v>0.25</v>
@@ -49130,7 +49143,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" s="90" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B69" s="91">
         <v>2</v>
@@ -49138,7 +49151,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" s="90" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B70" s="91">
         <v>0</v>
@@ -49146,7 +49159,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" s="90" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B71" s="91">
         <v>1</v>
@@ -49154,7 +49167,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" s="90" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B72" s="91">
         <v>0.25</v>
@@ -49162,7 +49175,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" s="90" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B73" s="91">
         <v>1</v>
@@ -49170,7 +49183,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" s="90" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B74" s="91">
         <v>0.25</v>
@@ -49178,7 +49191,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" s="90" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B75" s="91">
         <v>10</v>
@@ -49186,7 +49199,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" s="90" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B76" s="91">
         <v>13</v>
@@ -49194,7 +49207,7 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" s="90" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B77" s="91">
         <v>5</v>
@@ -49202,7 +49215,7 @@
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" s="90" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B78" s="91">
         <v>2.25</v>
@@ -49210,7 +49223,7 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" s="90" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B79" s="91">
         <v>2</v>
@@ -49218,7 +49231,7 @@
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" s="90" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B80" s="91">
         <v>2.75</v>
@@ -49226,7 +49239,7 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" s="90" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B81" s="91">
         <v>2</v>
@@ -49234,7 +49247,7 @@
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" s="90" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B82" s="91">
         <v>2</v>
@@ -49242,7 +49255,7 @@
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" s="90" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B83" s="91">
         <v>4</v>
@@ -49250,7 +49263,7 @@
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" s="90" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B84" s="91">
         <v>4.5</v>
@@ -49258,7 +49271,7 @@
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" s="90" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B85" s="91">
         <v>1</v>
@@ -49266,7 +49279,7 @@
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" s="90" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B86" s="91">
         <v>0</v>
@@ -49274,7 +49287,7 @@
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A87" s="90" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B87" s="91">
         <v>2</v>
@@ -49282,7 +49295,7 @@
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A88" s="90" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B88" s="91">
         <v>2.5</v>
@@ -49290,7 +49303,7 @@
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A89" s="90" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B89" s="91">
         <v>2</v>
@@ -49298,7 +49311,7 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A90" s="90" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B90" s="91">
         <v>3</v>
@@ -49306,7 +49319,7 @@
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A91" s="90" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B91" s="91">
         <v>5</v>
@@ -49314,7 +49327,7 @@
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A92" s="90" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B92" s="91">
         <v>3.75</v>
@@ -49322,7 +49335,7 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A93" s="90" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="B93" s="91">
         <v>4</v>
@@ -49330,7 +49343,7 @@
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A94" s="90" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B94" s="91">
         <v>5.5</v>
@@ -49338,7 +49351,7 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A95" s="90" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B95" s="91">
         <v>2</v>
@@ -49346,7 +49359,7 @@
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A96" s="90" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B96" s="91">
         <v>0</v>
@@ -49354,7 +49367,7 @@
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A97" s="90" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="B97" s="91">
         <v>1</v>
@@ -49362,7 +49375,7 @@
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A98" s="90" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B98" s="91">
         <v>3</v>
@@ -49370,7 +49383,7 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A99" s="90" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="B99" s="91">
         <v>1</v>
@@ -49378,7 +49391,7 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A100" s="90" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B100" s="91">
         <v>0.5</v>
@@ -49386,7 +49399,7 @@
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A101" s="90" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B101" s="91">
         <v>2</v>
@@ -49394,7 +49407,7 @@
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A102" s="90" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="B102" s="91">
         <v>2.5</v>
@@ -49402,7 +49415,7 @@
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A103" s="90" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B103" s="91">
         <v>1</v>
@@ -49410,7 +49423,7 @@
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A104" s="90" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B104" s="91">
         <v>0.5</v>
@@ -49418,7 +49431,7 @@
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A105" s="90" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B105" s="91">
         <v>1</v>
@@ -49426,7 +49439,7 @@
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A106" s="90" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B106" s="91">
         <v>1</v>
@@ -49434,7 +49447,7 @@
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A107" s="90" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B107" s="91">
         <v>4</v>
@@ -49442,7 +49455,7 @@
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A108" s="90" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B108" s="91">
         <v>10</v>
@@ -49450,7 +49463,7 @@
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A109" s="90" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B109" s="91">
         <v>5</v>
@@ -49458,7 +49471,7 @@
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A110" s="90" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="B110" s="91">
         <v>8</v>
@@ -49466,7 +49479,7 @@
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A111" s="90" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B111" s="91">
         <v>2</v>
@@ -49474,7 +49487,7 @@
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A112" s="90" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B112" s="91">
         <v>3</v>
@@ -49482,7 +49495,7 @@
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A113" s="90" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="B113" s="91">
         <v>2</v>
@@ -49490,7 +49503,7 @@
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A114" s="90" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B114" s="91">
         <v>5</v>
@@ -49498,7 +49511,7 @@
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A115" s="90" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B115" s="91">
         <v>6</v>
@@ -49506,7 +49519,7 @@
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A116" s="90" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="B116" s="91">
         <v>7.5</v>
@@ -49514,7 +49527,7 @@
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A117" s="90" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B117" s="91">
         <v>5</v>
@@ -49522,7 +49535,7 @@
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A118" s="90" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B118" s="91">
         <v>6</v>
@@ -49530,7 +49543,7 @@
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A119" s="90" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B119" s="91">
         <v>5</v>
@@ -49538,7 +49551,7 @@
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A120" s="90" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B120" s="91">
         <v>6.5</v>
@@ -49546,7 +49559,7 @@
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A121" s="90" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B121" s="91">
         <v>1</v>
@@ -49554,7 +49567,7 @@
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A122" s="90" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B122" s="91">
         <v>0.5</v>
@@ -49562,7 +49575,7 @@
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A123" s="90" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B123" s="91">
         <v>1</v>
@@ -49570,7 +49583,7 @@
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A124" s="90" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="B124" s="91">
         <v>1</v>
@@ -49578,7 +49591,7 @@
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A125" s="90" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B125" s="91">
         <v>1</v>
@@ -49586,7 +49599,7 @@
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A126" s="90" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B126" s="91">
         <v>3</v>
@@ -49594,7 +49607,7 @@
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A127" s="90" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B127" s="91">
         <v>3</v>
@@ -49602,7 +49615,7 @@
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A128" s="90" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B128" s="91">
         <v>1</v>
@@ -49610,7 +49623,7 @@
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A129" s="90" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B129" s="91">
         <v>1</v>
@@ -49618,7 +49631,7 @@
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A130" s="90" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B130" s="91">
         <v>2</v>
@@ -49626,7 +49639,7 @@
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A131" s="90" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B131" s="91">
         <v>14</v>
@@ -49634,7 +49647,7 @@
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A132" s="90" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B132" s="91">
         <v>19</v>
@@ -49650,7 +49663,7 @@
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A134" s="90" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B134" s="91">
         <v>7</v>
@@ -49682,7 +49695,7 @@
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A138" s="90" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B138" s="91">
         <v>40</v>
@@ -49698,7 +49711,7 @@
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A140" s="90" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="B140" s="91">
         <v>45</v>
@@ -49714,7 +49727,7 @@
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A142" s="90" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B142" s="91" t="b">
         <v>0</v>
@@ -49730,7 +49743,7 @@
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A144" s="90" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B144" s="91" t="b">
         <v>0</v>

</xml_diff>